<commit_message>
works euphoria and new dash
</commit_message>
<xml_diff>
--- a/docs/DECISIONS.xlsx
+++ b/docs/DECISIONS.xlsx
@@ -31,7 +31,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -105,6 +105,10 @@
     <font>
       <name val="Arial"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="7">
@@ -222,7 +226,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -304,6 +308,12 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -828,7 +838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="26" customWidth="1" style="12" min="1" max="1"/>
@@ -976,6 +986,219 @@
       <c r="C10" s="15" t="inlineStr">
         <is>
           <t>Thesis ethics sec 8.3.2 rationale: public pseudonymous identifiers used solely as node ids; no private data collected. Desk decision so live data keeps building one shared record.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="31" t="inlineStr">
+        <is>
+          <t>How the tab is READ - display decisions (2026-07-27 re-cut, after the desk said 'I still dont get it')</t>
+        </is>
+      </c>
+      <c r="B12" s="31" t="n"/>
+      <c r="C12" s="31" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>What ships</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>Class and reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>Section ORDER: exhibits first, board fourth (2026-07-27)</t>
+        </is>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>The tab opens with what the panel is PUSHING (bubble chart), then week by week, then who is behind one name, and only then the board of authors; the map and the two contrarian boards follow. It used to open with a list of usernames.</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>DESK DECISION. A PM does not trade a list of accounts, they trade positioning - so the board sits under the exhibits it is the evidence for. No computation changed; ordering only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="18" t="inlineStr">
+        <is>
+          <t>Unit: influence 0-100 instead of the raw composite (2026-07-27)</t>
+        </is>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>influence_index(board) = 100 x composite / composite.max(); the real store's max is 0.9854740019093133. The raw min-max composite is no longer printed anywhere on the tab, nor is the HIGH-tier cut (&gt;=0.66).</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
+        <is>
+          <t>DERIVED, and rank-identical. A positive rescaling cannot reorder anything, so no conclusion moved. Reason for the change is measured desk feedback: '0.987' printed next to a tier boundary reads as an accuracy, which it is not.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="18" t="inlineStr">
+        <is>
+          <t>Unit: backing as a SHARE of the room's conviction (2026-07-27)</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>backing_share = 100 x weighted_voices / sum(weighted_voices), bounded 0-100 and additive. Measured 30d cross-section, 51 names: MSFT 26.10%, ADBE 7.05, FICO 4.82, INTU 4.04, MELI 3.58, tail STRC 0.17.</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>DERIVED. A bare sum ('3.42') has no unit and cannot be compared between two windows or two names; a share can be spoken aloud, is immune to the long tail, and sums to a checkable 100.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="inlineStr">
+        <is>
+          <t>REJECTED: backing as a MULTIPLE of the median name, and the A1 analogy WITHDRAWN (2026-07-27)</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>backing_ratio = weighted / median(weighted) was built, measured and removed. Week to 2026-06-28: 163 names, median backing 0.24, so MSFT printed 141x. Weekly maxima 141x / 41x / 2.7x / 14x / 26x at 30d and 171x at 90d; with authors=None the median is exactly 0 and every ratio returned NaN.</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>REJECTED ON DATA. It was justified as mirroring the euphoria detector's A1 convention ('2x its own 120d median'). That argument is formally withdrawn: A1 anchors a name to ITS OWN history, a stable reference, whereas the median NAME in a cross-section is a ticker mentioned once by one person. Kept in this register because it was a recorded encoding decision before it was a rejected one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="18" t="inlineStr">
+        <is>
+          <t>The reference line is DERIVED, not chosen (2026-07-27)</t>
+        </is>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>even_share(n) = 100 / n - what each name would show if attention were split evenly. 2.0% across the 51 names in the 30d window, against MSFT's 26.1%, i.e. thirteen times an even share. Drawn per-week on the time chart, once on the cross-section. Replaces a 1.0x median hairline.</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="inlineStr">
+        <is>
+          <t>DERIVED from the count of names in the window, so there is no number to defend. This is the project's standing rule applied to a chart annotation: no arbitrary thresholds, including visual ones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="18" t="inlineStr">
+        <is>
+          <t>The share DENOMINATOR is fixed before any filter (2026-07-27)</t>
+        </is>
+      </c>
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>Both crowding_history (before the ticker filter) and fig_influence_bubbles (before head(top_n)) compute the share and the even-split line over the WHOLE window. The figure now receives the full digest plus top_n rather than an already-truncated frame.</t>
+        </is>
+      </c>
+      <c r="C19" s="19" t="inlineStr">
+        <is>
+          <t>BUG FIX, found by screenshotting the rendered chart. The chart printed MSFT at 29.5% (30 drawn names) while the KPI one row above printed 26.10% (51 names in the window), and the even line read 100/30 = 3.3% instead of 100/51 = 2.0%. One quantity cannot have two values on one screen. The dropped tail still counts in the denominator - that is the point of a share.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>Time panels use ALL recorded voices, not the top-N panel (2026-07-27)</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>The weekly tilt and per-name share history are computed over all 340 authors with &gt;=5 judged calls, independent of the panel_n slider. Top-25 weeks held 124, 25, 1, 23, 9 calls (the 1-call week is one name at 100% by definition) against 733, 404, 23, 98, 155 calls over 14-171 names for the full pool.</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="inlineStr">
+        <is>
+          <t>DERIVED from what a time series IS: a series whose population changes when a display slider moves is not comparable week to week. Measured counts are recorded here because they are the reason, not an illustration of it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>Thin weeks are ENCODED, never gated (2026-07-27)</t>
+        </is>
+      </c>
+      <c r="B21" s="19" t="inlineStr">
+        <is>
+          <t>Tilt-marker area is proportional to n_calls (sizemode='area', sizeref=2.0*cmax/20^2, sizemin=4). No week is dropped and no minimum call count exists.</t>
+        </is>
+      </c>
+      <c r="C21" s="19" t="inlineStr">
+        <is>
+          <t>Standing project rule: encode evidence, do not gate on it. A minimum-calls filter would be exactly the arbitrary threshold the desk has ruled out; a small dot says 'thin week' honestly and lets the reader decide.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>Label de-collision: the ONLY pixel-level rule on this project (2026-07-27)</t>
+        </is>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>dashboard._thin_labels suppresses a ticker label only when its box overlaps an already-placed one in BOTH directions; the weekly chart instead NUDGES end-of-line names apart as annotations. Gaps derived from geometry: 13px = one 10pt line box at 1.3 leading, 30px = a four-character ticker's width. Greedy in descending y; ties resolve to the earlier (better-backed) row.</t>
+        </is>
+      </c>
+      <c r="C22" s="19" t="inlineStr">
+        <is>
+          <t>PERMITTED because it is a rule about INK, not about DATA: every point is still drawn, still hovers, and still appears in the exact-numbers table, so nothing decides which names MATTER. Fenced by five unit tests in TestChartLabelLayout so it stays the only one. Triggered by INTU (4.04%) and MELI (3.58%) sitting 0.46pp = ~9px apart when a 10pt label needs 13px, and by MSTR/ADBE both ending near 0.3% as one illegible smear.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>REMOVED: fig_consensus (2026-07-27)</t>
+        </is>
+      </c>
+      <c r="B23" s="19" t="inlineStr">
+        <is>
+          <t>The stand-alone consensus bar chart is deleted. It plotted the same per-ticker consensus the bubble chart carries on its x-axis, with the bubble chart's y-axis folded into bar opacity - its own docstring said so.</t>
+        </is>
+      </c>
+      <c r="C23" s="19" t="inlineStr">
+        <is>
+          <t>Redundant exhibit. Its ENCODING decision is retained deliberately (bar length = direction, bar fade = weight of evidence, because bar length saturates at three agreeing voices) so the reasoning survives the chart, per the standing rule that anything used for a decision is recorded even after deletion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>REMOVED FROM DISPLAY: per-author hit rate (2026-07-27)</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>No hit rate is shown for any individual author anywhere on the tab; the board shows influence 0-100 and each author's tickers. The stored hit_rate column in author_scores.parquet is UNCHANGED and a schema test asserts it, and analytics/influence.py still computes it.</t>
+        </is>
+      </c>
+      <c r="C24" s="19" t="inlineStr">
+        <is>
+          <t>DESK DECISION ('dont include hit rate for users just show their influence and their stock tickers'), and it agrees with the measured limitation: per-author hit rates at n&gt;=5 judged calls are too thin to read as skill, and the cohort split shows the record does not generalise to unseen authors anyway.</t>
         </is>
       </c>
     </row>
@@ -995,7 +1218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="13" min="1" max="1"/>
@@ -1151,17 +1374,17 @@
       </c>
       <c r="B9" s="29" t="inlineStr">
         <is>
-          <t>STANDING EXPERIMENT: store is live-only and seeds on the first update_data.py run; NB05 re-renders from the real store each run. Harness validated on a schema-faithful synthetic fixture (deleted after use).</t>
+          <t>CONCLUDED 2026-07-27. Store matured (5,071 authors with &gt;=1 judged call; 107k accounts / 259k reply edges raw); notebook 05 executed clean and its verdict now feeds the dashboard's influence tab.</t>
         </is>
       </c>
       <c r="C9" s="29" t="inlineStr">
         <is>
-          <t>Forward record from inception - no backfill (desk decision).</t>
+          <t>Supersedes the STANDING EXPERIMENT status: the maturity criterion below was met (237 positives under the shipped label regime).</t>
         </is>
       </c>
       <c r="D9" s="29" t="inlineStr">
         <is>
-          <t>NB05 asserts store presence with instructions</t>
+          <t>notebooks/05_influence_users_model.ipynb; docs/research/nb05_influence.json</t>
         </is>
       </c>
     </row>
@@ -1184,6 +1407,226 @@
       <c r="D10" s="29" t="inlineStr">
         <is>
           <t>NB05 verdict cell</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="29" t="inlineStr">
+        <is>
+          <t>Model bank (final)</t>
+        </is>
+      </c>
+      <c r="B11" s="29" t="inlineStr">
+        <is>
+          <t>Eight architectures per thesis 6.1: random floor | logit | mlp | label_prop | gcn_lite | sage_lite | mixhop_lite | h2gcn_lite. GAT deliberately NOT ported.</t>
+        </is>
+      </c>
+      <c r="C11" s="29" t="inlineStr">
+        <is>
+          <t>GAT's attention must LEARN per-edge weights; ~250 positives cannot support it, so mixhop_lite is the named small-data stand-in. Refusing a layer we cannot train is itself the decision.</t>
+        </is>
+      </c>
+      <c r="D11" s="29" t="inlineStr">
+        <is>
+          <t>notebooks/05 section 6 tournament; influence_ml.py FULL bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="29" t="inlineStr">
+        <is>
+          <t>Label regime shipped</t>
+        </is>
+      </c>
+      <c r="B12" s="29" t="inlineStr">
+        <is>
+          <t>'softened' (237 positives). Strict = 25 positives (not powered); prevalence = 354.</t>
+        </is>
+      </c>
+      <c r="C12" s="29" t="inlineStr">
+        <is>
+          <t>The strictest definition that clears the &gt;=130-positive maturity bar. All three regimes reported side by side (thesis 7.1.2 labelling sensitivity).</t>
+        </is>
+      </c>
+      <c r="D12" s="29" t="inlineStr">
+        <is>
+          <t>notebooks/05 section 4; nb05_influence.json label_regimes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>SHIPPED model</t>
+        </is>
+      </c>
+      <c r="B13" s="29" t="inlineStr">
+        <is>
+          <t>logit on the 17-feature FULL_BANK. AP 0.0977 +/- 0.0242 vs random floor 0.0467; AUROC 0.6681; pooled precision 0.1176 (thesis SAGE: 0.140).</t>
+        </is>
+      </c>
+      <c r="C13" s="29" t="inlineStr">
+        <is>
+          <t>Adoption ladder under the paired 10-seed AP rule: random-&gt;logit +0.0464, CI [+0.0334,+0.0593], 10/10 seeds. Parsimony then stops there.</t>
+        </is>
+      </c>
+      <c r="D13" s="29" t="inlineStr">
+        <is>
+          <t>notebooks/05 section 7; assert shipped == influence_ml.BEST_MODEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="29" t="inlineStr">
+        <is>
+          <t>Every GRAPH layer REJECTED</t>
+        </is>
+      </c>
+      <c r="B14" s="29" t="inlineStr">
+        <is>
+          <t>mixhop +0.0011 CI [-0.0063,+0.0085]; sage_lite -0.0035; h2gcn -0.0078 CI [-0.0130,-0.0026] (significantly WORSE); gcn -0.0132; mlp -0.0326.</t>
+        </is>
+      </c>
+      <c r="C14" s="29" t="inlineStr">
+        <is>
+          <t>ci_lo &gt; 0 or the floor ships. No graph rung's interval cleared zero; one was significantly negative.</t>
+        </is>
+      </c>
+      <c r="D14" s="29" t="inlineStr">
+        <is>
+          <t>notebooks/05 section 7 adoption ladder</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>WHY the graph fails (measured)</t>
+        </is>
+      </c>
+      <c r="B15" s="29" t="inlineStr">
+        <is>
+          <t>Positive-class node homophily 0.0948 vs negative 0.9628 (thesis: 0.08 / 0.93). DICE perturbation RAISES AP: 0.1031 -&gt; 0.1528 -&gt; 0.1671 -&gt; 0.1884 -&gt; 0.2063 at 0/10/20/30/50% corruption, while accuracy falls 0.9343 -&gt; 0.8883. Random rewiring only mildly degrades (-&gt; 0.0978).</t>
+        </is>
+      </c>
+      <c r="C15" s="29" t="inlineStr">
+        <is>
+          <t>Good callers do not cluster, so message-passing averages their signal away - the diagnosis is measured, not asserted, and it replicates the thesis's direction (7.2).</t>
+        </is>
+      </c>
+      <c r="D15" s="29" t="inlineStr">
+        <is>
+          <t>notebooks/05 sections 3.6, 11, 12; nb05_influence.json homophily / perturbation</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>Circularity priced and REFUSED</t>
+        </is>
+      </c>
+      <c r="B16" s="29" t="inlineStr">
+        <is>
+          <t>mean_conf and stance_sd excluded (SCORE_ADJACENT). Including them lifts AP 0.1004 -&gt; 0.1987: mean_diff +0.0983, CI [+0.0834,+0.1132], 10/10 seeds.</t>
+        </is>
+      </c>
+      <c r="C16" s="29" t="inlineStr">
+        <is>
+          <t>mean_conf is an arithmetic factor of its own target. The cost of honesty is recorded rather than quietly avoided.</t>
+        </is>
+      </c>
+      <c r="D16" s="29" t="inlineStr">
+        <is>
+          <t>notebooks/05 section 5 circularity audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="29" t="inlineStr">
+        <is>
+          <t>Multiple-comparison discipline</t>
+        </is>
+      </c>
+      <c r="B17" s="29" t="inlineStr">
+        <is>
+          <t>Bonferroni within a round: 6 pre-stated bank candidates -&gt; conf 1 - 0.05/6 = 0.99167. One re-test round only, declared before the round ran. ADOPTED: NULL.</t>
+        </is>
+      </c>
+      <c r="C17" s="29" t="inlineStr">
+        <is>
+          <t>Of the six, only 'drop behavioural family' cleared zero at 95% (+0.0076, CI [+0.0023,+0.0128]); it did not survive correction.</t>
+        </is>
+      </c>
+      <c r="D17" s="29" t="inlineStr">
+        <is>
+          <t>notebooks/05 section 11.1; nb05_influence.json bonferroni</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="29" t="inlineStr">
+        <is>
+          <t>Significance</t>
+        </is>
+      </c>
+      <c r="B18" s="29" t="inlineStr">
+        <is>
+          <t>200-permutation label shuffle: AP 0.1257 vs null mean 0.0521, null p95 0.0705 -&gt; p = 0.005 (the reportable floor at 200 draws).</t>
+        </is>
+      </c>
+      <c r="C18" s="29" t="inlineStr">
+        <is>
+          <t>Thesis-style permutation test; the floor is stated as a floor, not rounded to 0.</t>
+        </is>
+      </c>
+      <c r="D18" s="29" t="inlineStr">
+        <is>
+          <t>notebooks/05 section 14</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="29" t="inlineStr">
+        <is>
+          <t>DECISIVE limitation: no generalisation</t>
+        </is>
+      </c>
+      <c r="B19" s="29" t="inlineStr">
+        <is>
+          <t>On a tenure/cohort split (unseen authors) the shipped model sits AT the random floor: logit AP 0.0461 vs random 0.0483 (lift -0.046); sage_lite 0.0410 (lift -0.150).</t>
+        </is>
+      </c>
+      <c r="C19" s="29" t="inlineStr">
+        <is>
+          <t>The one thing a model would be FOR - scoring a newcomer before they have a record - is exactly what it cannot do. Not a tuning gap; a stated negative result.</t>
+        </is>
+      </c>
+      <c r="D19" s="29" t="inlineStr">
+        <is>
+          <t>notebooks/05 section 15 cohort split</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="29" t="inlineStr">
+        <is>
+          <t>Consequence for the product</t>
+        </is>
+      </c>
+      <c r="B20" s="29" t="inlineStr">
+        <is>
+          <t>The dashboard's influence tab ranks authors by their MEASURED composite and is labelled INFORMATION ONLY; the model ships as a research exhibit, not a scorer. Nothing on the tab feeds the euphoria level or the GET IN / GET OUT alerts.</t>
+        </is>
+      </c>
+      <c r="C20" s="29" t="inlineStr">
+        <is>
+          <t>Follows directly from the cohort result above. Board shows authors with &gt;=5 judged calls (a record needs a record); the map covers the wider scored pool and says so.</t>
+        </is>
+      </c>
+      <c r="D20" s="29" t="inlineStr">
+        <is>
+          <t>dashboard.py influence tab; docs/ARCHITECTURE.md 8</t>
         </is>
       </c>
     </row>
@@ -1198,7 +1641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="30" customWidth="1" style="12" min="1" max="1"/>
@@ -1312,6 +1755,40 @@
       <c r="C8" s="15" t="inlineStr">
         <is>
           <t>Changes require NEW out-of-sample evidence, not re-runs of the same history.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>File retired: src/inflection.py (2026-07-27)</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>The FIRST take-off detector: smooth daily mentions, take the EWMA first derivative, and flag a day when that derivative exceeds mean + k*sigma. Rejected on principle, not on a metric - k is a free parameter with no derivation, so 'why k=2 and not 2.5?' has no answer. Its own docstring shows the flaw. Superseded by (a) analytics/euphoria.py, which ranks each name against ITS OWN history by percentile so the unit is calibrated per instrument rather than by a shared sigma multiple, and (b) analytics/euphoria_phases.py, which requires a sustained change in CONVEXITY instead of a single fast day - the fix for the 1-day XLE blip. The 'bull_inflection' FEATURE in dashboard.py is unrelated and stays.</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>REMOVED 2026-07-27 after a three-method reference audit (import regex, repo-relative path, bare filename) found zero references in 62 py files and 104 text files. sha256 5646a24fb1ab3abe... The idea it encodes is preserved here as the negative result that motivates per-name percentile ranking; no code depended on it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>File retired: helper/tune_thresholds.py (2026-07-27)</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>The BUY/SELL threshold tuner. Method worth keeping on the record: it grid-searched (SIG_K, SIG_MIN_SCORE, SIG_COOLDOWN), re-executed the real signal engine per combo via SIG_* env overrides so there was no reimplementation drift, scored each signal by SIGNED forward return, split the history into regime ERAS, and ranked combos by their WORST-era average - robustness first, so the winner is the combo that never falls apart rather than the one that aced a single mania. That worst-era rule is the provenance of the values still shipping in src/config.py: SIG_K=2.5, SIG_MIN_SCORE=4, SIG_MIN_SCORE_SELL=4, SIG_COOLDOWN_DAYS=21.</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>REMOVED 2026-07-27: it executes notebooks/10_trading_signals.ipynb, which no longer exists (notebooks are now 01-07), so the script fails on its first subprocess call - dead AND broken. Zero references by any of the three scan methods. sha256 51a8d0045dff09be... The four constants it produced remain live and are consumed by analytics/signals.py; this row is now their derivation of record, so they are not arbitrary numbers. To re-tune, port the worst-era protocol onto notebook 06/07.</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="30" customWidth="1" style="12" min="1" max="1"/>
@@ -1496,6 +1973,74 @@
       <c r="C11" s="19" t="inlineStr">
         <is>
           <t>Constants documented as ported (sheet 8); they set RELATIVE rankings, not absolute claims, so miscalibration degrades gracefully.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>Influence model does not generalise to new authors</t>
+        </is>
+      </c>
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>On a tenure/cohort split the influential-users model sits at the random floor for authors it has never seen (lift -0.046). Behaviour + graph position do NOT identify a good caller before they have a record.</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="inlineStr">
+        <is>
+          <t>Stated, not buried: the dashboard therefore ranks by the MEASURED record and labels the model a research exhibit. The tab is INFORMATION ONLY and feeds no signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="30" t="inlineStr">
+        <is>
+          <t>Reply graph is an active liability, not a weak feature</t>
+        </is>
+      </c>
+      <c r="B13" s="30" t="inlineStr">
+        <is>
+          <t>Corrupting the graph with DICE RAISES ranking quality (AP 0.1031 -&gt; 0.2063 at 50% corruption); positive-class homophily is 0.0948 vs 0.9628 for negatives.</t>
+        </is>
+      </c>
+      <c r="C13" s="30" t="inlineStr">
+        <is>
+          <t>Diagnosed rather than patched: every graph layer was rejected under the CI rule and the parsimony floor (logit) ships. The direction replicates the thesis (7.2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>Influence labels are score-derived, so circularity is a standing risk</t>
+        </is>
+      </c>
+      <c r="B14" s="30" t="inlineStr">
+        <is>
+          <t>The target is a tier of the same composite whose ingredients live in the store; two features (mean_conf, stance_sd) are arithmetic factors of it and would lift AP by +0.098 if used.</t>
+        </is>
+      </c>
+      <c r="C14" s="30" t="inlineStr">
+        <is>
+          <t>A named LEAKAGE blacklist plus a SCORE_ADJACENT exclusion, both asserted in tests; the audit that prices the excluded features is a permanent notebook section, so the cost is visible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="30" t="inlineStr">
+        <is>
+          <t>Influence store is forward-only and Reddit-only</t>
+        </is>
+      </c>
+      <c r="B15" s="30" t="inlineStr">
+        <is>
+          <t>The store begins at first pull - no backfill - so author records are short (median judged-call count is small) and the board needs &gt;=5 judged calls before it will rank anyone.</t>
+        </is>
+      </c>
+      <c r="C15" s="30" t="inlineStr">
+        <is>
+          <t>The bar is stated on the tab; records deepen with every comment pull, and matured calls are re-judged automatically. No decimal-level claim is made about any single author.</t>
         </is>
       </c>
     </row>
@@ -2328,7 +2873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="28" customWidth="1" style="12" min="1" max="1"/>
@@ -2479,10 +3024,10 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" s="13">
       <c r="A11" s="29" t="inlineStr">
         <is>
-          <t>Comments decoupled (2026-07-24)</t>
+          <t>Comments decoupled (2026-07-24) - SUPERSEDED 2026-07-27</t>
         </is>
       </c>
       <c r="B11" s="29" t="inlineStr">
@@ -2586,6 +3131,28 @@
       <c r="D15" s="29" t="inlineStr">
         <is>
           <t>episode_coherent_alerts + TestEpisodeCoherence (4 tests); dashboard draw_chart</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" s="13">
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>Comments BUDGETED back into the live pipeline (2026-07-27) - REVERSES row 11</t>
+        </is>
+      </c>
+      <c r="B16" s="29" t="inlineStr">
+        <is>
+          <t>update_data.py fetches comments on EVERY run again (--with-comments is now accepted and ignored; --skip-comments is the new opt-out), but under a measured PAGE ALLOWANCE instead of uncapped. src/pipeline_budget.py computes it as (600s desk ceiling - this machine's MEASURED non-fetch stage seconds) x 1 req/s, then splits it across subreddits in proportion to the days each one owes, with a one-page anti-starvation floor. Two self-measuring EWMA ledgers back it: pipeline_stage_times.json (stage costs) and reddit_comments_cost.json (pages/day per subreddit); both are gitignored because they measure ONE machine's speed. update_comments.py survives as the UNBUDGETED runner for backfills and long-gap catch-up, and its hand-written time ranges were replaced by a ledger-computed estimate.</t>
+        </is>
+      </c>
+      <c r="C16" s="29" t="inlineStr">
+        <is>
+          <t>WHY REVERSED: an influence board that rescores month-old comments is not a live board - row 11 optimised runtime at the cost of the tab's whole claim. WHY BUDGETED rather than simply switched back on: the cost was measured, not assumed. Intersecting comment-call rec_ids with reply_edges gives 12,010/417,208 = 2.879% call rate among comments, which against two independent months (403 and 414 comment-calls/day) implies ~14,000 comments/day = ~140 pages/day across the 17-sub panel - so a 7-day gap costs 16.3-16.8 min against the desk's ~10-min ceiling (caveat: the rate is measured on the edge-covered 48% of comment-calls). PIPELINE_BUDGET_S = 600 is the ONLY human-chosen number; alpha = 0.2 is DERIVED via the span identity 2/(N+1) with N = round(28/3.2) = 9, and the 5-day lookback is ceil(3.2)+1. REJECTED with reasons: a wall-clock stopwatch (data collected becomes a function of network luck, so no two runs compare and 'why did it stop there?' has no answer); parallel workers (W workers x 1s pauses = W req/s, breaking the politeness contract the project accepted when it chose a free public API); uniform window narrowing (penalises quiet subreddits to subsidise loud ones); per-subreddit yield ranking (the store has no subreddit column). The one legitimate speedup shipped: a Pacer sleeping the REMAINDER of the second instead of a flat second after each round-trip - 28% dead time removed at an unchanged request rate (261ms vs 360ms over 6 requests). Hitting a cap sets completed = False so the watermark does NOT advance: deferral, never loss - the board is never silently partial, only ever less fresh. Consequence the desk accepted: run the pipeline ~2x a week (the measured cadence is 3.32 days, i.e. what one allowance buys).</t>
+        </is>
+      </c>
+      <c r="D16" s="29" t="inlineStr">
+        <is>
+          <t>src/pipeline_budget.py (allocate/allowance_pages/non_fetch_seconds); src/config.py COMMENT INGESTION BUDGET block; ingestion/fetch_reddit_comments.py Pacer + --max-pages; fetch_all.py --comment-pages; update_data.py stage timing; PARAMETER_REGISTER Class 7; ARCHITECTURE 3.1b + 3.1b-i; RESEARCH_REPORT changelog 2026-07-27 (o). Verified: 75 tests pass, real run wrote the ledger and the allowance self-corrected 449 -&gt; 465 pages, plus two no-network stub tests (cap/watermark/ledger semantics; all three fetch_all hand-off paths).</t>
         </is>
       </c>
     </row>
@@ -3838,7 +4405,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="13" min="1" max="1"/>
@@ -4184,6 +4751,72 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="29" t="inlineStr">
+        <is>
+          <t>Improvement campaign: NOTHING adopted (2026-07-24, NB07)</t>
+        </is>
+      </c>
+      <c r="B18" s="29" t="inlineStr">
+        <is>
+          <t>Four pre-registered challengers vs the shipped desk configuration (adoption rule pre-stated: more captures, FAs not higher, paired cluster gain CI excluding zero): per-kind thresholds REJECTED (cap 23 vs 24 on unmatched years, though FA halved 39-&gt;16 - WATCH item); logistic-weighted score REJECTED by parsimony (30 vs 24 captures but gain CI [-1,+11] touches zero - WATCH item, auto re-test at year rollover); smoothing sweep w in {1,3,5,7,10,14}: no window dominates w=7; Western-Electric run rules k&gt;1: dominated by the smoothed single crossing.</t>
+        </is>
+      </c>
+      <c r="C18" s="29" t="inlineStr">
+        <is>
+          <t>The shipped configuration sits at the measured frontier. Watch items re-test automatically at the next --research pass under the same rule.</t>
+        </is>
+      </c>
+      <c r="D18" s="29" t="inlineStr">
+        <is>
+          <t>NB07 part B; nb07_performance_battery.json; RESEARCH_REPORT 6.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="29" t="inlineStr">
+        <is>
+          <t>Clustering-as-conviction REJECTED as exit criterion (2026-07-24, NB07)</t>
+        </is>
+      </c>
+      <c r="B19" s="29" t="inlineStr">
+        <is>
+          <t>The desk's 'buy-buy-buy / sell-sell-sell in a tight window' hypothesis, both forms: per-instrument intensity (trigger days in trailing 21d cooldown; STRONG = 2+ days) - cliff-30 rate 52.9% vs 55.9% single-day, uplift CI [-21pp,+22pp] straddles zero; cross-market breadth (share of names in GET OUT within 7d, top decile) - basket fwd-21d not separable at 90% (block bootstrap). A second GET OUT inside an episode is the same sell, not more sell.</t>
+        </is>
+      </c>
+      <c r="C19" s="29" t="inlineStr">
+        <is>
+          <t>The exit criterion remains the GET OUT alert itself; the cooldown + smoothed trigger already absorb repetition. The standing warning remains the danger-state band (NB06).</t>
+        </is>
+      </c>
+      <c r="D19" s="29" t="inlineStr">
+        <is>
+          <t>NB07 part C; RESEARCH_REPORT 6.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="29" t="inlineStr">
+        <is>
+          <t>Performance battery adopted into the research record (2026-07-24, NB07)</t>
+        </is>
+      </c>
+      <c r="B20" s="29" t="inlineStr">
+        <is>
+          <t>Literature-grounded metrics added: PR/F1/MCC at the operating point (Davis &amp; Goadrich; Chicco &amp; Jurman), delay-vs-FA frontier (Page 1954), MacKinlay CAR with cluster CIs, reliability diagram (Murphy &amp; Winkler), Grinold-Kahn IC, overlay Sharpe/Sortino (descriptive). The positive daily IC (+0.11) is recorded as PROOF the detector is an episode alarm, not daily alpha - a defense point, not a defect.</t>
+        </is>
+      </c>
+      <c r="C20" s="29" t="inlineStr">
+        <is>
+          <t>Desk asked for more metrics based on the research literature; every measure names its source in NB07 and the report references section.</t>
+        </is>
+      </c>
+      <c r="D20" s="29" t="inlineStr">
+        <is>
+          <t>NB07 part A; RESEARCH_REPORT 6.9 + references 8-14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
cleaned dashboard and new presentation
</commit_message>
<xml_diff>
--- a/docs/DECISIONS.xlsx
+++ b/docs/DECISIONS.xlsx
@@ -11,17 +11,18 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Motivation &amp; Aim" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. Literature" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. Data &amp; Architecture" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Detector Design" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Validation" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. Ablation" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. ML Challenger" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7b. Phases Study (Onset)" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. Influence Tracker" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8b. Influence ML Model" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. Legacy Decisions" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10. Limitations" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11. Next Steps" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12. References" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3b. Pipeline &amp; Cadence" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Detector Design" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Validation" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. Ablation" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. ML Challenger" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7b. Phases Study (Onset)" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. Influence Tracker" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8b. Influence ML Model" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="9. Legacy Decisions" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10. Limitations" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11. Next Steps" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12. References" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -31,7 +32,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -113,8 +114,25 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF1F3864"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -150,8 +168,13 @@
         <fgColor rgb="00D9E2F3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F3864"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -218,6 +241,14 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -229,7 +260,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -322,6 +353,28 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -843,6 +896,429 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" style="13" min="1" max="1"/>
+    <col width="52" customWidth="1" style="13" min="2" max="2"/>
+    <col width="46" customWidth="1" style="13" min="3" max="3"/>
+    <col width="40" customWidth="1" style="13" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>7b. Euphoria START detection - the July-2026 phases study (notebooks 01-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B3" s="28" t="inlineStr">
+        <is>
+          <t>Decision / result</t>
+        </is>
+      </c>
+      <c r="C3" s="28" t="inlineStr">
+        <is>
+          <t>Derivation (no arbitrary numbers)</t>
+        </is>
+      </c>
+      <c r="D3" s="28" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t>Aim</t>
+        </is>
+      </c>
+      <c r="B4" s="29" t="inlineStr">
+        <is>
+          <t>Detect the START of GME-scale euphoria episodes from the crowd alone, sparingly; plus confirm the TOP detector.</t>
+        </is>
+      </c>
+      <c r="C4" s="29" t="inlineStr">
+        <is>
+          <t>Extends the July-2026 re-aim; crowd-only hard rule unchanged (price = ground truth + scoring only).</t>
+        </is>
+      </c>
+      <c r="D4" s="29" t="inlineStr">
+        <is>
+          <t>notebooks/01-04; analytics/euphoria_phases.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="29" t="inlineStr">
+        <is>
+          <t>Episode ground truth</t>
+        </is>
+      </c>
+      <c r="B5" s="29" t="inlineStr">
+        <is>
+          <t>Boom-bust arc trough-&gt;peak-&gt;bust from the EXISTING peak rules G1-G3; trough = the 120d low G2 already measures the boom from.</t>
+        </is>
+      </c>
+      <c r="C5" s="29" t="inlineStr">
+        <is>
+          <t>No new fitted quantity: every threshold inherited from the validated top study.</t>
+        </is>
+      </c>
+      <c r="D5" s="29" t="inlineStr">
+        <is>
+          <t>NB01: 333 episodes, 126 onset-detectable, 136 top-detectable</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>Onset hit window</t>
+        </is>
+      </c>
+      <c r="B6" s="29" t="inlineStr">
+        <is>
+          <t>[trough, trough+45d], CAPPED at the peak; mid-rally alerts = LATE (neither hit nor false).</t>
+        </is>
+      </c>
+      <c r="C6" s="29" t="inlineStr">
+        <is>
+          <t>45d mirrors the existing FA horizon in score_alerts; cap prevents post-top alerts counting as 'caught the start'. Desk decision, recorded before results.</t>
+        </is>
+      </c>
+      <c r="D6" s="29" t="inlineStr">
+        <is>
+          <t>NB01 register; test_onset_window_capped_at_peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="29" t="inlineStr">
+        <is>
+          <t>Feature bank (locked)</t>
+        </is>
+      </c>
+      <c r="B7" s="29" t="inlineStr">
+        <is>
+          <t>attention_accel, hype_ratio, bull_inflection, influx_speed, attention_convexity.</t>
+        </is>
+      </c>
+      <c r="C7" s="29" t="inlineStr">
+        <is>
+          <t>Every window derived from existing constants (ROLL=7, 28d E-windows, 14d fade window, 120d hype baseline). source_breadth REJECTED: coverage-regime artifact (X/StockTwits exist only from 2026).</t>
+        </is>
+      </c>
+      <c r="D7" s="29" t="inlineStr">
+        <is>
+          <t>NB02 battery: per-feature AUROC + cluster-bootstrap CIs, ablation, perturbation</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>Tournament winner</t>
+        </is>
+      </c>
+      <c r="B8" s="29" t="inlineStr">
+        <is>
+          <t>RULES (unweighted bank mean, coverage + above-median-attention gates). GBM tied on AP but not outside the bootstrap CI -&gt; parsimony; MLP finished below random.</t>
+        </is>
+      </c>
+      <c r="C8" s="29" t="inlineStr">
+        <is>
+          <t>Criterion pre-stated: AP ranking (thesis 6.2.3), must beat random on AP+AUROC, parsimony CI rule; FA budget derived from the incumbent's accepted 0.23/instr-yr.</t>
+        </is>
+      </c>
+      <c r="D8" s="29" t="inlineStr">
+        <is>
+          <t>NB03: rules AP 0.098 vs random 0.072; top task: rules AP 0.286 vs random 0.204</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>Validated record</t>
+        </is>
+      </c>
+      <c r="B9" s="29" t="inlineStr">
+        <is>
+          <t>29/125 detectable onsets captured (23%), 21 late, 169 FA = 0.348/instr-yr (ABOVE the 0.23 budget - stated cost).</t>
+        </is>
+      </c>
+      <c r="C9" s="29" t="inlineStr">
+        <is>
+          <t>Walk-forward, thresholds from past years only; both denominators always reported.</t>
+        </is>
+      </c>
+      <c r="D9" s="29" t="inlineStr">
+        <is>
+          <t>NB04: median entry 17d after trough, 66d of rally still ahead</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="29" t="inlineStr">
+        <is>
+          <t>Label sensitivity</t>
+        </is>
+      </c>
+      <c r="B10" s="29" t="inlineStr">
+        <is>
+          <t>Capture rate flat across softened(20/40)/standard(25/50)/hardened(30/60) boom labels: 22.4%, 23.2%, 22.1%.</t>
+        </is>
+      </c>
+      <c r="C10" s="29" t="inlineStr">
+        <is>
+          <t>Thesis 7.1.2 port: conclusions must survive labelling perturbation.</t>
+        </is>
+      </c>
+      <c r="D10" s="29" t="inlineStr">
+        <is>
+          <t>NB03 sensitivity table</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="29" t="inlineStr">
+        <is>
+          <t>Trading translation</t>
+        </is>
+      </c>
+      <c r="B11" s="29" t="inlineStr">
+        <is>
+          <t>REJECTED for both ONSET-&gt;BUY and TOP-&gt;SELL under the pre-stated criterion (n&gt;=30, beats same-instrument 20d baseline, CI excludes 0).</t>
+        </is>
+      </c>
+      <c r="C11" s="29" t="inlineStr">
+        <is>
+          <t>Same treatment as the retired BUY/SELL engine; evidence retained.</t>
+        </is>
+      </c>
+      <c r="D11" s="29" t="inlineStr">
+        <is>
+          <t>NB04: onset diff -0.63% CI [-0.0151, 0.0026]; top diff -1.55% CI [-0.0563, 0.0263]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="29" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="B12" s="29" t="inlineStr">
+        <is>
+          <t>New 'Start / End radar' tab: STARTING and ENDING panes, each split Themes | Single names; only names alerted within the 21d cooldown; record printed on the pane.</t>
+        </is>
+      </c>
+      <c r="C12" s="29" t="inlineStr">
+        <is>
+          <t>Sparse by design - an empty pane is the radar working.</t>
+        </is>
+      </c>
+      <c r="D12" s="29" t="inlineStr">
+        <is>
+          <t>dashboard.py t_phase; AppTest 0 exceptions</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>Price-assisted END gate (2026-07-24)</t>
+        </is>
+      </c>
+      <c r="B13" s="29" t="inlineStr">
+        <is>
+          <t>PASSED all pre-stated conditions: G2 boom thresholds as a live prerequisite -&gt; capture 16-&gt;26 detectable tops (matched years), AP 0.286-&gt;0.435, FAs 44-&gt;41, capture-gain CI [+3.5pp,+13pp]. Offered as labelled second signal; claim becomes 'crowd + chart'.</t>
+        </is>
+      </c>
+      <c r="C13" s="29" t="inlineStr">
+        <is>
+          <t>The gate reuses the ground-truth boom definition on trailing prices - no new constant, no look-ahead.</t>
+        </is>
+      </c>
+      <c r="D13" s="29" t="inlineStr">
+        <is>
+          <t>NB03 commissioned-test section</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="29" t="inlineStr">
+        <is>
+          <t>Combined price+crowd ALERT bank (2026-07-24)</t>
+        </is>
+      </c>
+      <c r="B14" s="29" t="inlineStr">
+        <is>
+          <t>REJECTED under pre-stated criterion: 65% cliff-30 hit rate indistinguishable from its own 62% candidate-day baseline (CI includes 0). Smoothed-trigger evidence retained: FA 31-&gt;24 at equal capture, median trigger run 6-&gt;8d.</t>
+        </is>
+      </c>
+      <c r="C14" s="29" t="inlineStr">
+        <is>
+          <t>The alert layer cannot out-predict its own danger state; its job is timing the peak, which it does (median 8d lead).</t>
+        </is>
+      </c>
+      <c r="D14" s="29" t="inlineStr">
+        <is>
+          <t>NB06 desk-signal study</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>DANGER STATE shipped (2026-07-24)</t>
+        </is>
+      </c>
+      <c r="B15" s="29" t="inlineStr">
+        <is>
+          <t>The candidacy state (A1 2x hype AND G2 boom) validated as the standing drop-warning: cliff-30 = 62% in-state vs 19% ordinary, uplift CI [+28pp,+50pp]. Rendered as the amber band on every terminal price panel.</t>
+        </is>
+      </c>
+      <c r="C15" s="29" t="inlineStr">
+        <is>
+          <t>Pure composition of two existing constants; the single most actionable statistic of the project for the PM use case.</t>
+        </is>
+      </c>
+      <c r="D15" s="29" t="inlineStr">
+        <is>
+          <t>NB06; dashboard danger band; PARAMETER_REGISTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>DESK CONFIGURATION adopted: GET OUT (2026-07-24)</t>
+        </is>
+      </c>
+      <c r="B16" s="29" t="inlineStr">
+        <is>
+          <t>Boom-gated END rules + 7d-smoothed (ROLL) trigger. Walk-forward: capture 24/122 detectable tops, FA 39 (0.195/instr-yr), AP 0.449 (raw gate 0.435), median warning 8d before the peak. Smoothing adopted by pre-stated rule (AP not lower AND FAs not higher); 2-capture cost recorded. Frozen live threshold 0.630 (budget rule, full prior years).</t>
+        </is>
+      </c>
+      <c r="C16" s="29" t="inlineStr">
+        <is>
+          <t>The desk lifted the crowd-only rule for a labelled SECOND family ('use both price and social media - I want a better hit rate') and demanded no one-day blips. Candidacy = A1 hype AND G2 boom (existing constants only).</t>
+        </is>
+      </c>
+      <c r="D16" s="29" t="inlineStr">
+        <is>
+          <t>NB06 adopted-configuration section; euphoria_desk_report.json; euphoria_phases.py §6</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="29" t="inlineStr">
+        <is>
+          <t>DESK CONFIGURATION adopted: GET IN (2026-07-24)</t>
+        </is>
+      </c>
+      <c r="B17" s="29" t="inlineStr">
+        <is>
+          <t>Phase-aware onset (end-stage days - A1∧A2∧A3-persistence - excluded from candidacy) + 7d smoothing. Adjacency (START within 21d before an END) 20→2, LATE 21→10, FA 169→124; capture cost 29→20 of 125 RECORDED. Frozen live threshold 0.848. OVERRULES the earlier utility-rule rejection of the phase-aware variant as an explicit desk decision.</t>
+        </is>
+      </c>
+      <c r="C17" s="29" t="inlineStr">
+        <is>
+          <t>The desk stated three times that a START landing on an END destroys PM trust - adjacency is the binding constraint, so it overrules raw capture. Selection rule pre-stated in NB06; drift guard pins notebook == production.</t>
+        </is>
+      </c>
+      <c r="D17" s="29" t="inlineStr">
+        <is>
+          <t>NB06; euphoria_desk_report.json; PARAMETER_REGISTER class 5; dashboard GET IN/GET OUT banners</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="29" t="inlineStr">
+        <is>
+          <t>Improvement campaign: NOTHING adopted (2026-07-24, NB07)</t>
+        </is>
+      </c>
+      <c r="B18" s="29" t="inlineStr">
+        <is>
+          <t>Four pre-registered challengers vs the shipped desk configuration (adoption rule pre-stated: more captures, FAs not higher, paired cluster gain CI excluding zero): per-kind thresholds REJECTED (cap 23 vs 24 on unmatched years, though FA halved 39-&gt;16 - WATCH item); logistic-weighted score REJECTED by parsimony (30 vs 24 captures but gain CI [-1,+11] touches zero - WATCH item, auto re-test at year rollover); smoothing sweep w in {1,3,5,7,10,14}: no window dominates w=7; Western-Electric run rules k&gt;1: dominated by the smoothed single crossing.</t>
+        </is>
+      </c>
+      <c r="C18" s="29" t="inlineStr">
+        <is>
+          <t>The shipped configuration sits at the measured frontier. Watch items re-test automatically at the next --research pass under the same rule.</t>
+        </is>
+      </c>
+      <c r="D18" s="29" t="inlineStr">
+        <is>
+          <t>NB07 part B; nb07_performance_battery.json; RESEARCH_REPORT 6.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="29" t="inlineStr">
+        <is>
+          <t>Clustering-as-conviction REJECTED as exit criterion (2026-07-24, NB07)</t>
+        </is>
+      </c>
+      <c r="B19" s="29" t="inlineStr">
+        <is>
+          <t>The desk's 'buy-buy-buy / sell-sell-sell in a tight window' hypothesis, both forms: per-instrument intensity (trigger days in trailing 21d cooldown; STRONG = 2+ days) - cliff-30 rate 52.9% vs 55.9% single-day, uplift CI [-21pp,+22pp] straddles zero; cross-market breadth (share of names in GET OUT within 7d, top decile) - basket fwd-21d not separable at 90% (block bootstrap). A second GET OUT inside an episode is the same sell, not more sell.</t>
+        </is>
+      </c>
+      <c r="C19" s="29" t="inlineStr">
+        <is>
+          <t>The exit criterion remains the GET OUT alert itself; the cooldown + smoothed trigger already absorb repetition. The standing warning remains the danger-state band (NB06).</t>
+        </is>
+      </c>
+      <c r="D19" s="29" t="inlineStr">
+        <is>
+          <t>NB07 part C; RESEARCH_REPORT 6.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="29" t="inlineStr">
+        <is>
+          <t>Performance battery adopted into the research record (2026-07-24, NB07)</t>
+        </is>
+      </c>
+      <c r="B20" s="29" t="inlineStr">
+        <is>
+          <t>Literature-grounded metrics added: PR/F1/MCC at the operating point (Davis &amp; Goadrich; Chicco &amp; Jurman), delay-vs-FA frontier (Page 1954), MacKinlay CAR with cluster CIs, reliability diagram (Murphy &amp; Winkler), Grinold-Kahn IC, overlay Sharpe/Sortino (descriptive). The positive daily IC (+0.11) is recorded as PROOF the detector is an episode alarm, not daily alpha - a defense point, not a defect.</t>
+        </is>
+      </c>
+      <c r="C20" s="29" t="inlineStr">
+        <is>
+          <t>Desk asked for more metrics based on the research literature; every measure names its source in NB07 and the report references section.</t>
+        </is>
+      </c>
+      <c r="D20" s="29" t="inlineStr">
+        <is>
+          <t>NB07 part A; RESEARCH_REPORT 6.9 + references 8-14</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
@@ -1323,7 +1799,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1746,7 +2222,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1900,258 +2376,6 @@
       <c r="C10" s="15" t="inlineStr">
         <is>
           <t>REMOVED 2026-07-27: it executes notebooks/10_trading_signals.ipynb, which no longer exists (notebooks are now 01-07), so the script fails on its first subprocess call - dead AND broken. Zero references by any of the three scan methods. sha256 51a8d0045dff09be... The four constants it produced remain live and are consumed by analytics/signals.py; this row is now their derivation of record, so they are not arbitrary numbers. To re-tune, port the worst-era protocol onto notebook 06/07.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
-  </mergeCells>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="30" customWidth="1" style="12" min="1" max="1"/>
-    <col width="52" customWidth="1" style="12" min="2" max="2"/>
-    <col width="44" customWidth="1" style="12" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="25.5" customHeight="1" s="13">
-      <c r="A1" s="14" t="inlineStr">
-        <is>
-          <t>10. Limitations &amp; risks (the examiner's sheet)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="13">
-      <c r="A3" s="17" t="inlineStr">
-        <is>
-          <t>Limitation</t>
-        </is>
-      </c>
-      <c r="B3" s="17" t="inlineStr">
-        <is>
-          <t>Honest statement</t>
-        </is>
-      </c>
-      <c r="C3" s="17" t="inlineStr">
-        <is>
-          <t>Mitigation / response</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="35.05" customHeight="1" s="13">
-      <c r="A4" s="20" t="inlineStr">
-        <is>
-          <t>Coverage cliffs</t>
-        </is>
-      </c>
-      <c r="B4" s="15" t="inlineStr">
-        <is>
-          <t>2023-25 archive coverage is thin -&gt; ZERO detectable peaks there; the detector is blind, not wrong, in those eras - and 44+34 real peaks sit outside its reach.</t>
-        </is>
-      </c>
-      <c r="C4" s="15" t="inlineStr">
-        <is>
-          <t>Both denominators always reported; the comment backfill (~10x volume) is the direct fix (sheet 11).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="35.05" customHeight="1" s="13">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Reddit-only capture cost</t>
-        </is>
-      </c>
-      <c r="B5" s="19" t="inlineStr">
-        <is>
-          <t>23% of detectable vs 46% for the price-assisted variant: the chart carries real information the desk chose to give up.</t>
-        </is>
-      </c>
-      <c r="C5" s="19" t="inlineStr">
-        <is>
-          <t>A deliberate, documented trade for the clean claim; the price-assisted harness remains in git history if the desk ever re-decides.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="35.05" customHeight="1" s="13">
-      <c r="A6" s="20" t="inlineStr">
-        <is>
-          <t>Small event counts</t>
-        </is>
-      </c>
-      <c r="B6" s="15" t="inlineStr">
-        <is>
-          <t>17 captures / 74 detectable peaks - single events move rates by ~1.4pp; per-year splits are noisier still.</t>
-        </is>
-      </c>
-      <c r="C6" s="15" t="inlineStr">
-        <is>
-          <t>No decimal-level claims; ablation read at the big-movement level only; walk-forward (never pooled) evaluation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="35.05" customHeight="1" s="13">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t>Sentiment label noise</t>
-        </is>
-      </c>
-      <c r="B7" s="19" t="inlineStr">
-        <is>
-          <t>VADER+lexicon mislabels sarcasm and implicit calls; the thesis measured ~15-20% forecast-extraction error even with an LLM [1].</t>
-        </is>
-      </c>
-      <c r="C7" s="19" t="inlineStr">
-        <is>
-          <t>Errors average out at 28d aggregation and author-level scoring (same argument as the thesis); LLM extraction is the named upgrade (sheet 11).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="35.05" customHeight="1" s="13">
-      <c r="A8" s="20" t="inlineStr">
-        <is>
-          <t>Threshold at grid edge</t>
-        </is>
-      </c>
-      <c r="B8" s="15" t="inlineStr">
-        <is>
-          <t>Recent years pick threshold 85 = the grid maximum - the utility landscape wants conservatism, so the effective trigger is the fade discount.</t>
-        </is>
-      </c>
-      <c r="C8" s="15" t="inlineStr">
-        <is>
-          <t>Documented; grid deliberately NOT extended after seeing results (that would be fitting the grid to the test).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="35.05" customHeight="1" s="13">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t>2021 undertrained</t>
-        </is>
-      </c>
-      <c r="B9" s="19" t="inlineStr">
-        <is>
-          <t>2021's threshold is the do-no-harm default (its training years pre-date price history).</t>
-        </is>
-      </c>
-      <c r="C9" s="19" t="inlineStr">
-        <is>
-          <t>Extending prices to 2017 (one command) gives 2018-20 real peaks -&gt; 2021 gets trained; numbers auto-refresh.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="23.85" customHeight="1" s="13">
-      <c r="A10" s="20" t="inlineStr">
-        <is>
-          <t>Survivorship &amp; curation</t>
-        </is>
-      </c>
-      <c r="B10" s="15" t="inlineStr">
-        <is>
-          <t>Deleted posts vanish from live fetches; authors curate their history (thesis flags the same bias [1]).</t>
-        </is>
-      </c>
-      <c r="C10" s="15" t="inlineStr">
-        <is>
-          <t>Arctic Shift archives shortly after posting (partial); the ingest ledger keeps first-seen records once fetched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="35.05" customHeight="1" s="13">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t>One-subreddit thesis, many-subreddit desk</t>
-        </is>
-      </c>
-      <c r="B11" s="19" t="inlineStr">
-        <is>
-          <t>The thesis validated on r/CryptoMarkets; our transfer of its constants (shrinkage strengths, tier cutoff, filters) assumes they travel.</t>
-        </is>
-      </c>
-      <c r="C11" s="19" t="inlineStr">
-        <is>
-          <t>Constants documented as ported (sheet 8); they set RELATIVE rankings, not absolute claims, so miscalibration degrades gracefully.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="30" t="inlineStr">
-        <is>
-          <t>Influence model does not generalise to new authors</t>
-        </is>
-      </c>
-      <c r="B12" s="30" t="inlineStr">
-        <is>
-          <t>On a tenure/cohort split the influential-users model sits at the random floor for authors it has never seen (lift -0.046). Behaviour + graph position do NOT identify a good caller before they have a record.</t>
-        </is>
-      </c>
-      <c r="C12" s="30" t="inlineStr">
-        <is>
-          <t>Stated, not buried: the dashboard therefore ranks by the MEASURED record and labels the model a research exhibit. The tab is INFORMATION ONLY and feeds no signal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="30" t="inlineStr">
-        <is>
-          <t>Reply graph is an active liability, not a weak feature</t>
-        </is>
-      </c>
-      <c r="B13" s="30" t="inlineStr">
-        <is>
-          <t>Corrupting the graph with DICE RAISES ranking quality (AP 0.1031 -&gt; 0.2063 at 50% corruption); positive-class homophily is 0.0948 vs 0.9628 for negatives.</t>
-        </is>
-      </c>
-      <c r="C13" s="30" t="inlineStr">
-        <is>
-          <t>Diagnosed rather than patched: every graph layer was rejected under the CI rule and the parsimony floor (logit) ships. The direction replicates the thesis (7.2).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="30" t="inlineStr">
-        <is>
-          <t>Influence labels are score-derived, so circularity is a standing risk</t>
-        </is>
-      </c>
-      <c r="B14" s="30" t="inlineStr">
-        <is>
-          <t>The target is a tier of the same composite whose ingredients live in the store; two features (mean_conf, stance_sd) are arithmetic factors of it and would lift AP by +0.098 if used.</t>
-        </is>
-      </c>
-      <c r="C14" s="30" t="inlineStr">
-        <is>
-          <t>A named LEAKAGE blacklist plus a SCORE_ADJACENT exclusion, both asserted in tests; the audit that prices the excluded features is a permanent notebook section, so the cost is visible.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="30" t="inlineStr">
-        <is>
-          <t>Influence store is forward-only and Reddit-only</t>
-        </is>
-      </c>
-      <c r="B15" s="30" t="inlineStr">
-        <is>
-          <t>The store begins at first pull - no backfill - so author records are short (median judged-call count is small) and the board needs &gt;=5 judged calls before it will rank anyone.</t>
-        </is>
-      </c>
-      <c r="C15" s="30" t="inlineStr">
-        <is>
-          <t>The bar is stated on the tab; records deepen with every comment pull, and matured calls are re-judged automatically. No decimal-level claim is made about any single author.</t>
         </is>
       </c>
     </row>
@@ -2171,137 +2395,239 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="34" customWidth="1" style="12" min="1" max="1"/>
-    <col width="56" customWidth="1" style="12" min="2" max="2"/>
-    <col width="34" customWidth="1" style="12" min="3" max="3"/>
+    <col width="30" customWidth="1" style="12" min="1" max="1"/>
+    <col width="52" customWidth="1" style="12" min="2" max="2"/>
+    <col width="44" customWidth="1" style="12" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="25.5" customHeight="1" s="13">
       <c r="A1" s="14" t="inlineStr">
         <is>
-          <t>11. Next steps, ranked by expected impact</t>
+          <t>10. Limitations &amp; risks (the examiner's sheet)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="13">
       <c r="A3" s="17" t="inlineStr">
         <is>
-          <t>Step</t>
+          <t>Limitation</t>
         </is>
       </c>
       <c r="B3" s="17" t="inlineStr">
         <is>
-          <t>Why it is the biggest lever</t>
+          <t>Honest statement</t>
         </is>
       </c>
       <c r="C3" s="17" t="inlineStr">
         <is>
-          <t>Command / owner</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="57.45" customHeight="1" s="13">
+          <t>Mitigation / response</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="35.05" customHeight="1" s="13">
       <c r="A4" s="20" t="inlineStr">
         <is>
-          <t>1. Comment backfill -&gt; aggregates</t>
+          <t>Coverage cliffs</t>
         </is>
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>Comments are ~10x post volume and feed EVERY euphoria ingredient; 2022-25 become detectable, capture should recover toward (and possibly past) the price-assisted 46% WITHOUT touching the Reddit-only rule. The ML challenger auto-re-runs on the richer data under the already-stated criterion.</t>
+          <t>2023-25 archive coverage is thin -&gt; ZERO detectable peaks there; the detector is blind, not wrong, in those eras - and 44+34 real peaks sit outside its reach.</t>
         </is>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
-          <t>python ingestion/fetch_reddit_comments.py --backfill &lt;half-years&gt;; then fold into aggregates (external machine --full)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="57.45" customHeight="1" s="13">
+          <t>Both denominators always reported; the comment backfill (~10x volume) is the direct fix (sheet 11).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="35.05" customHeight="1" s="13">
       <c r="A5" s="18" t="inlineStr">
         <is>
-          <t>2. Prices to 2017</t>
+          <t>Reddit-only capture cost</t>
         </is>
       </c>
       <c r="B5" s="19" t="inlineStr">
         <is>
-          <t>Turns 2018-20 into real training AND test years (2018 vol shock, 2020 covid tops); 2021 stops being undertrained.</t>
+          <t>23% of detectable vs 46% for the price-assisted variant: the chart carries real information the desk chose to give up.</t>
         </is>
       </c>
       <c r="C5" s="19" t="inlineStr">
         <is>
-          <t>PowerShell: $env:PIPELINE_START_DATE="2017-01-01"; python pull_bloomberg_prices.py; then python -m analytics.run_analytics --what euphoria</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="23.85" customHeight="1" s="13">
+          <t>A deliberate, documented trade for the clean claim; the price-assisted harness remains in git history if the desk ever re-decides.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="35.05" customHeight="1" s="13">
       <c r="A6" s="20" t="inlineStr">
         <is>
-          <t>3. Influence store: nothing to run (live-only)</t>
+          <t>Small event counts</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Desk decision, July 2026: the store builds itself from live pulls - created from nothing on the first update_data.py run, extended on every later one, with recent calls re-judged automatically as their 20d windows mature. The two dashboards share it via git.</t>
+          <t>17 captures / 74 detectable peaks - single events move rates by ~1.4pp; per-year splits are noisier still.</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>automatic (python update_data.py)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="23.85" customHeight="1" s="13">
+          <t>No decimal-level claims; ablation read at the big-movement level only; walk-forward (never pooled) evaluation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="35.05" customHeight="1" s="13">
       <c r="A7" s="18" t="inlineStr">
         <is>
-          <t>4. Forward out-of-sample record</t>
+          <t>Sentiment label noise</t>
         </is>
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>The frozen rules + daily snapshots mean every week from now is TRUE out-of-sample - the only evidence that survives an examiner.</t>
+          <t>VADER+lexicon mislabels sarcasm and implicit calls; the thesis measured ~15-20% forecast-extraction error even with an LLM [1].</t>
         </is>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>Automatic; review monthly</t>
+          <t>Errors average out at 28d aggregation and author-level scoring (same argument as the thesis); LLM extraction is the named upgrade (sheet 11).</t>
         </is>
       </c>
     </row>
     <row r="8" ht="35.05" customHeight="1" s="13">
       <c r="A8" s="20" t="inlineStr">
         <is>
-          <t>5. LLM call extraction (thesis upgrade)</t>
+          <t>Threshold at grid edge</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Replace VADER stance with structured forecast extraction (direction/asset/horizon/confidence) - the thesis's biggest quality step (macro-F1 0.78, kappa 0.76) [1].</t>
+          <t>Recent years pick threshold 85 = the grid maximum - the utility landscape wants conservatism, so the effective trigger is the fade discount.</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>Future work - needs a funded API budget</t>
+          <t>Documented; grid deliberately NOT extended after seeing results (that would be fitting the grid to the test).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="35.05" customHeight="1" s="13">
       <c r="A9" s="18" t="inlineStr">
         <is>
-          <t>6. Graph features INTO euphoria</t>
+          <t>2021 undertrained</t>
         </is>
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>New-author influx and reply-graph growth as euphoria features (crowd composition, not just size) - the thesis's structural signals applied to the timing problem.</t>
+          <t>2021's threshold is the do-no-harm default (its training years pre-date price history).</t>
         </is>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>Future work - needs comments folded into the aggregate contract first</t>
+          <t>Extending prices to 2017 (one command) gives 2018-20 real peaks -&gt; 2021 gets trained; numbers auto-refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="23.85" customHeight="1" s="13">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>Survivorship &amp; curation</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Deleted posts vanish from live fetches; authors curate their history (thesis flags the same bias [1]).</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>Arctic Shift archives shortly after posting (partial); the ingest ledger keeps first-seen records once fetched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="35.05" customHeight="1" s="13">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>One-subreddit thesis, many-subreddit desk</t>
+        </is>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>The thesis validated on r/CryptoMarkets; our transfer of its constants (shrinkage strengths, tier cutoff, filters) assumes they travel.</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>Constants documented as ported (sheet 8); they set RELATIVE rankings, not absolute claims, so miscalibration degrades gracefully.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="30" t="inlineStr">
+        <is>
+          <t>Influence model does not generalise to new authors</t>
+        </is>
+      </c>
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>On a tenure/cohort split the influential-users model sits at the random floor for authors it has never seen (lift -0.046). Behaviour + graph position do NOT identify a good caller before they have a record.</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="inlineStr">
+        <is>
+          <t>Stated, not buried: the dashboard therefore ranks by the MEASURED record and labels the model a research exhibit. The tab is INFORMATION ONLY and feeds no signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="30" t="inlineStr">
+        <is>
+          <t>Reply graph is an active liability, not a weak feature</t>
+        </is>
+      </c>
+      <c r="B13" s="30" t="inlineStr">
+        <is>
+          <t>Corrupting the graph with DICE RAISES ranking quality (AP 0.1031 -&gt; 0.2063 at 50% corruption); positive-class homophily is 0.0948 vs 0.9628 for negatives.</t>
+        </is>
+      </c>
+      <c r="C13" s="30" t="inlineStr">
+        <is>
+          <t>Diagnosed rather than patched: every graph layer was rejected under the CI rule and the parsimony floor (logit) ships. The direction replicates the thesis (7.2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>Influence labels are score-derived, so circularity is a standing risk</t>
+        </is>
+      </c>
+      <c r="B14" s="30" t="inlineStr">
+        <is>
+          <t>The target is a tier of the same composite whose ingredients live in the store; two features (mean_conf, stance_sd) are arithmetic factors of it and would lift AP by +0.098 if used.</t>
+        </is>
+      </c>
+      <c r="C14" s="30" t="inlineStr">
+        <is>
+          <t>A named LEAKAGE blacklist plus a SCORE_ADJACENT exclusion, both asserted in tests; the audit that prices the excluded features is a permanent notebook section, so the cost is visible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="30" t="inlineStr">
+        <is>
+          <t>Influence store is forward-only and Reddit-only</t>
+        </is>
+      </c>
+      <c r="B15" s="30" t="inlineStr">
+        <is>
+          <t>The store begins at first pull - no backfill - so author records are short (median judged-call count is small) and the board needs &gt;=5 judged calls before it will rank anyone.</t>
+        </is>
+      </c>
+      <c r="C15" s="30" t="inlineStr">
+        <is>
+          <t>The bar is stated on the tab; records deepen with every comment pull, and matured calls are re-judged automatically. No decimal-level claim is made about any single author.</t>
         </is>
       </c>
     </row>
@@ -2316,6 +2642,156 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="34" customWidth="1" style="12" min="1" max="1"/>
+    <col width="56" customWidth="1" style="12" min="2" max="2"/>
+    <col width="34" customWidth="1" style="12" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25.5" customHeight="1" s="13">
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>11. Next steps, ranked by expected impact</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="13">
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B3" s="17" t="inlineStr">
+        <is>
+          <t>Why it is the biggest lever</t>
+        </is>
+      </c>
+      <c r="C3" s="17" t="inlineStr">
+        <is>
+          <t>Command / owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="57.45" customHeight="1" s="13">
+      <c r="A4" s="20" t="inlineStr">
+        <is>
+          <t>1. Comment backfill -&gt; aggregates</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Comments are ~10x post volume and feed EVERY euphoria ingredient; 2022-25 become detectable, capture should recover toward (and possibly past) the price-assisted 46% WITHOUT touching the Reddit-only rule. The ML challenger auto-re-runs on the richer data under the already-stated criterion.</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>python ingestion/fetch_reddit_comments.py --backfill &lt;half-years&gt;; then fold into aggregates (external machine --full)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="57.45" customHeight="1" s="13">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>2. Prices to 2017</t>
+        </is>
+      </c>
+      <c r="B5" s="19" t="inlineStr">
+        <is>
+          <t>Turns 2018-20 into real training AND test years (2018 vol shock, 2020 covid tops); 2021 stops being undertrained.</t>
+        </is>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>PowerShell: $env:PIPELINE_START_DATE="2017-01-01"; python pull_bloomberg_prices.py; then python -m analytics.run_analytics --what euphoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="23.85" customHeight="1" s="13">
+      <c r="A6" s="20" t="inlineStr">
+        <is>
+          <t>3. Influence store: nothing to run (live-only)</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Desk decision, July 2026: the store builds itself from live pulls - created from nothing on the first update_data.py run, extended on every later one, with recent calls re-judged automatically as their 20d windows mature. The two dashboards share it via git.</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>automatic (python update_data.py)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="23.85" customHeight="1" s="13">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>4. Forward out-of-sample record</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>The frozen rules + daily snapshots mean every week from now is TRUE out-of-sample - the only evidence that survives an examiner.</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>Automatic; review monthly</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="35.05" customHeight="1" s="13">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>5. LLM call extraction (thesis upgrade)</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>Replace VADER stance with structured forecast extraction (direction/asset/horizon/confidence) - the thesis's biggest quality step (macro-F1 0.78, kappa 0.76) [1].</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>Future work - needs a funded API budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="35.05" customHeight="1" s="13">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>6. Graph features INTO euphoria</t>
+        </is>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>New-author influx and reply-graph growth as euphoria features (crowd composition, not just size) - the thesis's structural signals applied to the timing problem.</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>Future work - needs comments folded into the aggregate contract first</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3357,11 +3833,255 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" style="13" min="1" max="1"/>
+    <col width="46" customWidth="1" style="13" min="2" max="2"/>
+    <col width="30" customWidth="1" style="13" min="3" max="3"/>
+    <col width="24" customWidth="1" style="13" min="4" max="4"/>
+    <col width="30" customWidth="1" style="13" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25.5" customHeight="1" s="13">
+      <c r="A1" s="40" t="inlineStr">
+        <is>
+          <t>3b. Pipeline &amp; Cadence - when a number is allowed to change, and who is allowed to change it</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="41" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="B3" s="41" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+      <c r="C3" s="41" t="inlineStr">
+        <is>
+          <t>Rationale</t>
+        </is>
+      </c>
+      <c r="D3" s="41" t="inlineStr">
+        <is>
+          <t>Parameter(s)</t>
+        </is>
+      </c>
+      <c r="E3" s="41" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="34" t="inlineStr">
+        <is>
+          <t>A LIVE RUN NEVER RE-SELECTS (2026-07-28)</t>
+        </is>
+      </c>
+      <c r="B4" s="35" t="inlineStr">
+        <is>
+          <t>update_data.py does not choose a model, re-select a threshold, or re-run the walk-forward, the ablation or the ML challenger. It refreshes data and scores it with the already-frozen winner, every time, so the run is one predictable job.</t>
+        </is>
+      </c>
+      <c r="C4" s="35" t="inlineStr">
+        <is>
+          <t>DESK DECISION: 'why does the update_data have to check what is the best model everytime? shouldnt it just used the already pre established best model? no need to show me the stats everytime.' The deeper reason is defensibility, not speed: re-fitting on every run makes the number on screen untraceable. Nothing on disk would describe how today's threshold differs from yesterday's, and a threshold nobody can reconstruct cannot be defended in a review.</t>
+        </is>
+      </c>
+      <c r="D4" s="35" t="inlineStr">
+        <is>
+          <t>None re-derived on a live run. The frozen record is data/processed/euphoria_desk_report.json.</t>
+        </is>
+      </c>
+      <c r="E4" s="35" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="34" t="inlineStr">
+        <is>
+          <t>THE ONE EXCEPTION: the bootstrap</t>
+        </is>
+      </c>
+      <c r="B5" s="35" t="inlineStr">
+        <is>
+          <t>A machine holding no frozen record at all derives one, once, before it can score anything.</t>
+        </is>
+      </c>
+      <c r="C5" s="35" t="inlineStr">
+        <is>
+          <t>You cannot score against a record that does not exist. This is the whole of the exception - it is not a fallback that can trigger on a machine that already has a record.</t>
+        </is>
+      </c>
+      <c r="D5" s="35" t="inlineStr">
+        <is>
+          <t>needs_research(stored) returns True only for `not stored or not stored.get('thresholds')`.</t>
+        </is>
+      </c>
+      <c r="E5" s="35" t="inlineStr">
+        <is>
+          <t>SHIPPED</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="34" t="inlineStr">
+        <is>
+          <t>TWO EXPLICIT WAYS TO RE-OPEN RESEARCH</t>
+        </is>
+      </c>
+      <c r="B6" s="35" t="inlineStr">
+        <is>
+          <t>`python -m analytics.run_analytics --what phases --research`, or `python update_data.py --full`.</t>
+        </is>
+      </c>
+      <c r="C6" s="35" t="inlineStr">
+        <is>
+          <t>Both are typed on purpose and never reached by drift. --full counts as research BECAUSE A BACKFILL REWRITES THE HISTORY THE THRESHOLDS WERE CHOSEN ON: scoring rebuilt history against thresholds fitted on the old history would be a silent lookahead.</t>
+        </is>
+      </c>
+      <c r="D6" s="35" t="inlineStr">
+        <is>
+          <t>--research forces re-derivation of thresholds and validation records.</t>
+        </is>
+      </c>
+      <c r="E6" s="35" t="inlineStr">
+        <is>
+          <t>SHIPPED</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="34" t="inlineStr">
+        <is>
+          <t>STALENESS IS REPORTED, NOT REPAIRED</t>
+        </is>
+      </c>
+      <c r="B7" s="35" t="inlineStr">
+        <is>
+          <t>When the frozen record stops at an earlier year than the data, the run prints ONE notice line and keeps scoring at the frozen threshold.</t>
+        </is>
+      </c>
+      <c r="C7" s="35" t="inlineStr">
+        <is>
+          <t>A live run in this state is legitimate - it is out-of-sample use, which is exactly what a walk-forward licenses. Refitting in January because a new year began does not make the threshold more correct; it makes it a moving target that no stored record describes. So the pipeline tells the desk to run the research pass rather than quietly doing it.</t>
+        </is>
+      </c>
+      <c r="D7" s="35" t="inlineStr">
+        <is>
+          <t>record_lags_data(stored, data_max_year) returns the newest covered year, else None.</t>
+        </is>
+      </c>
+      <c r="E7" s="35" t="inlineStr">
+        <is>
+          <t>SHIPPED</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="34" t="inlineStr">
+        <is>
+          <t>NO STATS PRINTED ON A LIVE RUN</t>
+        </is>
+      </c>
+      <c r="B8" s="35" t="inlineStr">
+        <is>
+          <t>Performance output belongs to the notebooks. The pipeline prints a data-coverage table, a window check, a run summary and the text-free safety-check verdict - operational facts, not research results.</t>
+        </is>
+      </c>
+      <c r="C8" s="35" t="inlineStr">
+        <is>
+          <t>Same principle as the dashboard's no-performance-metrics decision: the notebooks are the research record, the operational surfaces state conclusions. 'if i need to know the stats i will use th enotebooks.'</t>
+        </is>
+      </c>
+      <c r="D8" s="35" t="inlineStr">
+        <is>
+          <t>None.</t>
+        </is>
+      </c>
+      <c r="E8" s="35" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-07-28 - see sheet '4. Detector Design'</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="34" t="inlineStr">
+        <is>
+          <t>CADENCE and the RUN BUDGET</t>
+        </is>
+      </c>
+      <c r="B9" s="35" t="inlineStr">
+        <is>
+          <t>The pipeline is run roughly twice a week. A full refresh, influence included, must stay under about ten minutes.</t>
+        </is>
+      </c>
+      <c r="C9" s="35" t="inlineStr">
+        <is>
+          <t>Alex's answer when asked directly, plus 'not really a bounded time budget, but a full update of the dashboard (like weekly) running shouldnt take more than ~10 minutes'. The budget is expressed as a number the code can enforce rather than as an intention.</t>
+        </is>
+      </c>
+      <c r="D9" s="35" t="inlineStr">
+        <is>
+          <t>PIPELINE_BUDGET_S = 600 (src/config.py); ingestion budget in PARAMETER_REGISTER Class 7.</t>
+        </is>
+      </c>
+      <c r="E9" s="35" t="inlineStr">
+        <is>
+          <t>SHIPPED</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="34" t="inlineStr">
+        <is>
+          <t>POINTER CORRECTION - recorded because it was wrong in shipped source</t>
+        </is>
+      </c>
+      <c r="B10" s="35" t="inlineStr">
+        <is>
+          <t>analytics/euphoria.py promised this contract lived in DECISIONS.xlsx '2. Pipeline &amp; Cadence' and PARAMETER_REGISTER Class 6. Neither held it: sheet 2 is Literature, Class 6 is the influence tracker. This sheet and PARAMETER_REGISTER Class 9 were created to hold it, and the docstrings were repointed.</t>
+        </is>
+      </c>
+      <c r="C10" s="35" t="inlineStr">
+        <is>
+          <t>Renumbering the existing sheets and classes would have been the other option and was rejected: every other cross-reference in the repo - source docstrings, the research report, the decks - would have broken silently. Creating the missing sections costs nothing and breaks nothing.</t>
+        </is>
+      </c>
+      <c r="D10" s="35" t="inlineStr">
+        <is>
+          <t>analytics/euphoria.py::needs_research docstring, lines 788-789.</t>
+        </is>
+      </c>
+      <c r="E10" s="35" t="inlineStr">
+        <is>
+          <t>FIXED 2026-07-28</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="12" min="1" max="1"/>
@@ -3406,665 +4126,976 @@
       </c>
     </row>
     <row r="4" ht="23.85" customHeight="1" s="13">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="34" t="inlineStr">
         <is>
           <t>E1</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="35" t="inlineStr">
         <is>
           <t>Attention extremity: trailing pct-rank of the 7d mention share (vs the name's own last 365d).</t>
         </is>
       </c>
-      <c r="C4" s="15" t="inlineStr">
+      <c r="C4" s="35" t="inlineStr">
         <is>
           <t>You cannot be euphoric quietly [2].</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
+      <c r="D4" s="35" t="inlineStr">
         <is>
           <t>rank window 365d, min 180d</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr">
+      <c r="E4" s="35" t="inlineStr">
         <is>
           <t>Fixed a priori</t>
         </is>
       </c>
     </row>
     <row r="5" ht="57.45" customHeight="1" s="13">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="36" t="inlineStr">
         <is>
           <t>E2</t>
         </is>
       </c>
-      <c r="B5" s="19" t="inlineStr">
+      <c r="B5" s="37" t="inlineStr">
         <is>
           <t>Sustained bullishness: pct-rank of the 28d net-bullish share, x0 unless &gt;=75% of the last 28 POSTING days were net-bullish.</t>
         </is>
       </c>
-      <c r="C5" s="19" t="inlineStr">
+      <c r="C5" s="37" t="inlineStr">
         <is>
           <t>Desk hypothesis 1: weeks of one-way lean, not one loud day. Persistence over posting days: a zero-post day is 'no evidence', not 'not bullish'.</t>
         </is>
       </c>
-      <c r="D5" s="19" t="inlineStr">
+      <c r="D5" s="37" t="inlineStr">
         <is>
           <t>28d window, 75% persistence</t>
         </is>
       </c>
-      <c r="E5" s="19" t="inlineStr">
+      <c r="E5" s="37" t="inlineStr">
         <is>
           <t>Fixed a priori</t>
         </is>
       </c>
     </row>
     <row r="6" ht="23.85" customHeight="1" s="13">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="34" t="inlineStr">
         <is>
           <t>E3</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="35" t="inlineStr">
         <is>
           <t>Crowd influx: pct-rank of the 28d CHANGE in mention share.</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C6" s="35" t="inlineStr">
         <is>
           <t>The crowd is still arriving - late-stage contagion.</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="35" t="inlineStr">
         <is>
           <t>28d diff</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="E6" s="35" t="inlineStr">
         <is>
           <t>Fixed a priori</t>
         </is>
       </c>
     </row>
     <row r="7" ht="46.25" customHeight="1" s="13">
-      <c r="A7" s="18" t="inlineStr">
+      <c r="A7" s="36" t="inlineStr">
         <is>
           <t>E5</t>
         </is>
       </c>
-      <c r="B7" s="19" t="inlineStr">
+      <c r="B7" s="37" t="inlineStr">
         <is>
           <t>Super-exponential ATTENTION growth: pct-rank of positive convexity of log(1+mentions, 7d-smoothed) over a rolling 60d quadratic fit.</t>
         </is>
       </c>
-      <c r="C7" s="19" t="inlineStr">
+      <c r="C7" s="37" t="inlineStr">
         <is>
           <t>Sornette's bubble signature [3][4][7][8], applied to the crowd (Reddit-only rule): accelerating contagion must saturate.</t>
         </is>
       </c>
-      <c r="D7" s="19" t="inlineStr">
+      <c r="D7" s="37" t="inlineStr">
         <is>
           <t>60d fit window</t>
         </is>
       </c>
-      <c r="E7" s="19" t="inlineStr">
+      <c r="E7" s="37" t="inlineStr">
         <is>
           <t>Fixed a priori</t>
         </is>
       </c>
     </row>
     <row r="8" ht="23.85" customHeight="1" s="13">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="34" t="inlineStr">
         <is>
           <t>LEVEL</t>
         </is>
       </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="B8" s="35" t="inlineStr">
         <is>
           <t>EUPHORIA LEVEL = 100 x mean(E1, E2, E3, E5).</t>
         </is>
       </c>
-      <c r="C8" s="15" t="inlineStr">
+      <c r="C8" s="35" t="inlineStr">
         <is>
           <t>Equal weights - no fitted feature weights to overfit.</t>
         </is>
       </c>
-      <c r="D8" s="15" t="inlineStr">
+      <c r="D8" s="35" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E8" s="15" t="inlineStr">
+      <c r="E8" s="35" t="inlineStr">
         <is>
           <t>Fixed a priori</t>
         </is>
       </c>
     </row>
     <row r="9" ht="35.05" customHeight="1" s="13">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="36" t="inlineStr">
         <is>
           <t>E4 fade</t>
         </is>
       </c>
-      <c r="B9" s="19" t="inlineStr">
+      <c r="B9" s="37" t="inlineStr">
         <is>
           <t>Trigger sharpener: attention &gt;= 90th pct while the 14d bullish share change is NEGATIVE -&gt; alert threshold drops by 10 points.</t>
         </is>
       </c>
-      <c r="C9" s="19" t="inlineStr">
+      <c r="C9" s="37" t="inlineStr">
         <is>
           <t>Desk hypothesis 2: crowd maximal, mood rolling over - historically the LAST stage before the top.</t>
         </is>
       </c>
-      <c r="D9" s="19" t="inlineStr">
+      <c r="D9" s="37" t="inlineStr">
         <is>
           <t>discount 10 pts</t>
         </is>
       </c>
-      <c r="E9" s="19" t="inlineStr">
+      <c r="E9" s="37" t="inlineStr">
         <is>
           <t>Fixed a priori</t>
         </is>
       </c>
     </row>
     <row r="10" ht="23.85" customHeight="1" s="13">
-      <c r="A10" s="20" t="inlineStr">
+      <c r="A10" s="34" t="inlineStr">
         <is>
           <t>A0</t>
         </is>
       </c>
-      <c r="B10" s="15" t="inlineStr">
+      <c r="B10" s="35" t="inlineStr">
         <is>
           <t>Coverage gate: &gt;= 100 scored posts in the last 28d.</t>
         </is>
       </c>
-      <c r="C10" s="15" t="inlineStr">
+      <c r="C10" s="35" t="inlineStr">
         <is>
           <t>Percentile extremes on a handful of posts are noise wearing a costume.</t>
         </is>
       </c>
-      <c r="D10" s="15" t="inlineStr">
+      <c r="D10" s="35" t="inlineStr">
         <is>
           <t>100 posts</t>
         </is>
       </c>
-      <c r="E10" s="15" t="inlineStr">
+      <c r="E10" s="35" t="inlineStr">
         <is>
           <t>Fixed a priori</t>
         </is>
       </c>
     </row>
     <row r="11" ht="46.25" customHeight="1" s="13">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="36" t="inlineStr">
         <is>
           <t>A1</t>
         </is>
       </c>
-      <c r="B11" s="19" t="inlineStr">
+      <c r="B11" s="37" t="inlineStr">
         <is>
           <t>Hype prerequisite: 7d mention share &gt;= 2.0x its own trailing 120d MEDIAN.</t>
         </is>
       </c>
-      <c r="C11" s="19" t="inlineStr">
+      <c r="C11" s="37" t="inlineStr">
         <is>
           <t>'Something must go euphoric first' - measured in the crowd, never the chart. Median (not min) so the gate cannot be vacuous.</t>
         </is>
       </c>
-      <c r="D11" s="19" t="inlineStr">
+      <c r="D11" s="37" t="inlineStr">
         <is>
           <t>2.0x, 120d</t>
         </is>
       </c>
-      <c r="E11" s="19" t="inlineStr">
+      <c r="E11" s="37" t="inlineStr">
         <is>
           <t>Fixed a priori</t>
         </is>
       </c>
     </row>
     <row r="12" ht="23.85" customHeight="1" s="13">
-      <c r="A12" s="20" t="inlineStr">
+      <c r="A12" s="34" t="inlineStr">
         <is>
           <t>A2 / A2b</t>
         </is>
       </c>
-      <c r="B12" s="15" t="inlineStr">
+      <c r="B12" s="35" t="inlineStr">
         <is>
           <t>Attention &gt;= 90th pct AND E2 &gt; 0 as hard prerequisites.</t>
         </is>
       </c>
-      <c r="C12" s="15" t="inlineStr">
+      <c r="C12" s="35" t="inlineStr">
         <is>
           <t>Desk hypotheses 3 and 1 as gates, not just score components.</t>
         </is>
       </c>
-      <c r="D12" s="15" t="inlineStr">
+      <c r="D12" s="35" t="inlineStr">
         <is>
           <t>0.90</t>
         </is>
       </c>
-      <c r="E12" s="15" t="inlineStr">
+      <c r="E12" s="35" t="inlineStr">
         <is>
           <t>Fixed a priori</t>
         </is>
       </c>
     </row>
     <row r="13" ht="35.05" customHeight="1" s="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="36" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="B13" s="19" t="inlineStr">
+      <c r="B13" s="37" t="inlineStr">
         <is>
           <t>Level &gt;= threshold (or &gt;= threshold - 10 with fade active).</t>
         </is>
       </c>
-      <c r="C13" s="19" t="inlineStr">
+      <c r="C13" s="37" t="inlineStr">
         <is>
           <t>THE trigger.</t>
         </is>
       </c>
-      <c r="D13" s="19" t="inlineStr">
+      <c r="D13" s="37" t="inlineStr">
         <is>
           <t>threshold in {50..85}</t>
         </is>
       </c>
-      <c r="E13" s="19" t="inlineStr">
+      <c r="E13" s="37" t="inlineStr">
         <is>
           <t>FITTED - walk-forward only, past years only; conservative default when training is empty</t>
         </is>
       </c>
     </row>
     <row r="14" ht="23.85" customHeight="1" s="13">
-      <c r="A14" s="20" t="inlineStr">
+      <c r="A14" s="34" t="inlineStr">
         <is>
           <t>A4</t>
         </is>
       </c>
-      <c r="B14" s="15" t="inlineStr">
+      <c r="B14" s="35" t="inlineStr">
         <is>
           <t>Cooldown: one alert per name per 21 days.</t>
         </is>
       </c>
-      <c r="C14" s="15" t="inlineStr">
+      <c r="C14" s="35" t="inlineStr">
         <is>
           <t>One alert per episode - a manic month is one call, not twenty.</t>
         </is>
       </c>
-      <c r="D14" s="15" t="inlineStr">
+      <c r="D14" s="35" t="inlineStr">
         <is>
           <t>21d</t>
         </is>
       </c>
-      <c r="E14" s="15" t="inlineStr">
+      <c r="E14" s="35" t="inlineStr">
         <is>
           <t>Fixed a priori</t>
         </is>
       </c>
     </row>
     <row r="15" ht="46.25" customHeight="1" s="13">
-      <c r="A15" s="18" t="inlineStr">
+      <c r="A15" s="36" t="inlineStr">
         <is>
           <t>Judging</t>
         </is>
       </c>
-      <c r="B15" s="19" t="inlineStr">
+      <c r="B15" s="37" t="inlineStr">
         <is>
           <t>Alerts count only inside the judgeable window: price history exists at the alert AND for 45d after.</t>
         </is>
       </c>
-      <c r="C15" s="19" t="inlineStr">
+      <c r="C15" s="37" t="inlineStr">
         <is>
           <t>Pre-price-history alerts are PENDING, not false - scoring them as FAs was a measured bug (fixed July 2026).</t>
         </is>
       </c>
-      <c r="D15" s="19" t="inlineStr">
+      <c r="D15" s="37" t="inlineStr">
         <is>
           <t>45d</t>
         </is>
       </c>
-      <c r="E15" s="19" t="inlineStr">
+      <c r="E15" s="37" t="inlineStr">
         <is>
           <t>Fixed a priori</t>
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="34" t="n"/>
+      <c r="B16" s="35" t="n"/>
+      <c r="C16" s="35" t="n"/>
+      <c r="D16" s="35" t="n"/>
+      <c r="E16" s="35" t="n"/>
+    </row>
     <row r="17" ht="57.45" customHeight="1" s="13">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="38" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="B17" s="22" t="inlineStr">
+      <c r="B17" s="39" t="inlineStr">
         <is>
           <t>The one deliberate trade: an earlier variant also used price features (log-price convexity + a price-boom gate) and captured 46% of detectable peaks. The Reddit-only rule gives that up for the clean claim. The delta is quantified on sheet 5 and the recovery path on sheet 11.</t>
         </is>
       </c>
-      <c r="C17" s="22" t="n"/>
-      <c r="D17" s="22" t="n"/>
-      <c r="E17" s="22" t="n"/>
+      <c r="C17" s="39" t="n"/>
+      <c r="D17" s="39" t="n"/>
+      <c r="E17" s="39" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="34" t="n"/>
+      <c r="B18" s="35" t="n"/>
+      <c r="C18" s="35" t="n"/>
+      <c r="D18" s="35" t="n"/>
+      <c r="E18" s="35" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="32" t="inlineStr">
+      <c r="A19" s="34" t="inlineStr">
         <is>
           <t>GAUGE (display, 2026-07-27)</t>
         </is>
       </c>
-      <c r="B19" s="33" t="inlineStr">
+      <c r="B19" s="35" t="inlineStr">
         <is>
           <t>A speedometer above every theme and every ticker chart. Needle = the 7d-smoothed euphoria level (0-100) read at the last day of the selected window; delta = the same curve ROLL=7 days earlier; bands = calm below 76, warming 76-84, RED ZONE 85+. Wired inside draw_chart, which runs once per instrument in BOTH tabs, so 'for each theme / ticker' is structural rather than duplicated code.</t>
         </is>
       </c>
-      <c r="C19" s="33" t="inlineStr">
+      <c r="C19" s="35" t="inlineStr">
         <is>
           <t>DESK REQUEST, verbatim: 'a very clear speedometer thing for each graph (and showing the change) for each theme / ticker'. The construction constraint was that a dial is the most compressive exhibit on the project - a PM reads one number and one colour and acts - so it was built to introduce exactly ONE new number. The needle is not a new quantity (it is literally the object the lower panel already plots, so dial and chart cannot disagree - unit-tested) and the red edge is not a new number either (see next row).</t>
         </is>
       </c>
-      <c r="D19" s="33" t="inlineStr">
+      <c r="D19" s="35" t="inlineStr">
         <is>
           <t>needle = ROLL(7); bands from docs/research/gauge_zones.json</t>
         </is>
       </c>
-      <c r="E19" s="33" t="inlineStr">
+      <c r="E19" s="35" t="inlineStr">
         <is>
           <t>SHIPPED - 9 tests (84 -&gt; 93)</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="32" t="inlineStr">
+      <c r="A20" s="34" t="inlineStr">
         <is>
           <t>GAUGE RED EDGE = 85</t>
         </is>
       </c>
-      <c r="B20" s="33" t="inlineStr">
+      <c r="B20" s="35" t="inlineStr">
         <is>
           <t>Read at import time out of data/processed/euphoria_report.json's thresholds dict - the level the walk-forward already selected for the ENDING alert, which is 85 in every test year 2018-2026.</t>
         </is>
       </c>
-      <c r="C20" s="33" t="inlineStr">
+      <c r="C20" s="35" t="inlineStr">
         <is>
           <t>A gauge that chose its own red edge would be a SECOND, SOFTER THRESHOLD competing with the detector, and the dashboard would then hold two different opinions about when euphoria is dangerous. A unit test asserts equality with the report; notebook 06 asserts the walk-forward agreed across years, on the stated grounds that if it had NOT, a single red edge would be a fiction and the honest exhibit would be each year's own level.</t>
         </is>
       </c>
-      <c r="D20" s="33" t="inlineStr">
+      <c r="D20" s="35" t="inlineStr">
         <is>
           <t>85 (level units) - NOT a new constant</t>
         </is>
       </c>
-      <c r="E20" s="33" t="inlineStr">
+      <c r="E20" s="35" t="inlineStr">
         <is>
           <t>LEARNED (reused) - unit-tested against euphoria_report.json</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="32" t="inlineStr">
+      <c r="A21" s="34" t="inlineStr">
         <is>
           <t>GAUGE AMBER EDGE = 76</t>
         </is>
       </c>
-      <c r="B21" s="33" t="inlineStr">
+      <c r="B21" s="35" t="inlineStr">
         <is>
           <t>The lowest cut on a 2-point grid from 68 whose 95% PAIRED cluster-bootstrap lower bound on P(drop | level&gt;=L) - P(drop | level&lt;L) excludes zero under ALL FIVE seeds. Outcome graded is the desk's own '&lt;1 month' horizon, unchanged from the desk-signal study: does a fall of &gt;=10% over 7 days START within the next 30 days (implemented as a reversed rolling max; the last 30+7=37 days are NaN, because scoring an incomplete look-ahead as 'no drop' would bias the base rate down exactly at the live edge). Resampling unit is the INSTRUMENT, never the day.</t>
         </is>
       </c>
-      <c r="C21" s="33" t="inlineStr">
+      <c r="C21" s="35" t="inlineStr">
         <is>
           <t>THE ONE NEW NUMBER, and the route to it is the methodological point. (i) THE OBVIOUS TEST WAS THE WRONG TEST: comparing a 95% CI for P(drop | level&gt;=L) against a 95% CI for the base rate found NOTHING significant at any cut from 40 to 95. That is the overlapping-confidence-interval fallacy, not a null result - with 59 instruments both intervals are wide and overlap everywhere, and two overlapping intervals do not mean the difference is zero. Bootstrapping the DIFFERENCE (state minus not-state) on the SAME resampled instruments cancels the shared instrument-level noise and recovers a significant effect at every cut from 76 up. This first method ships nowhere; it is recorded here and in NB06's prose, with no code left behind. (ii) WHY NAMES AND NOT DAYS: adjacent days on one instrument are the same episode, so a day-level bootstrap would treat 4,000 days of one mania as 4,000 independent facts and report an interval several times too tight. (iii) WHY 76 AND NOT 74: the rule was stated before the grid was run, and cut 74 FLIPS SIGN across seeds (-0.0004, +0.0009, -0.0012, -0.0007, +0.0004) while cut 76 does not (+0.0045, +0.0060, +0.0049, +0.0034, +0.0046). A cut that changes sign with the random seed is not a parameter. Honest limitation recorded: this edge is selected in-sample on the full panel, not walk-forward - which is precisely why it colours a DISPLAY band and never fires a trigger.</t>
         </is>
       </c>
-      <c r="D21" s="33" t="inlineStr">
+      <c r="D21" s="35" t="inlineStr">
         <is>
           <t>76 (level units); grid 68-90 step 2, 5 seeds, 4,000 reps</t>
         </is>
       </c>
-      <c r="E21" s="33" t="inlineStr">
+      <c r="E21" s="35" t="inlineStr">
         <is>
           <t>LEARNED by a pre-stated rule - grid in gauge_zones.json</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="32" t="inlineStr">
+      <c r="A22" s="34" t="inlineStr">
         <is>
           <t>GAUGE - what each band is WORTH</t>
         </is>
       </c>
-      <c r="B22" s="33" t="inlineStr">
+      <c r="B22" s="35" t="inlineStr">
         <is>
           <t>Measured on 183,394 name-days / 59 instruments / 2017-06-29 to 2026-06-15. Base rate 23.3%. level&gt;=76: 26.9% (n=11,235, +3.9pp, CI [+0.6,+7.4]). level&gt;=85: 30.4% (n=4,203, +7.3pp [+2.1,+12.8]). Danger state alone (crowd 2x own median AND price boom): 53.8% (n=3,819, +31.2pp [+22.2,+40.1]). level&gt;=85 AND danger state: 71.4% (n=454, +48.2pp [+34.3,+59.5]).</t>
         </is>
       </c>
-      <c r="C22" s="33" t="inlineStr">
+      <c r="C22" s="35" t="inlineStr">
         <is>
           <t>THE DIAL ADMITS ITS OWN WEAKNESS ON ITS FACE. The level ALONE at the red edge is 30% against a 23% base rate - only ~1.3x. The level TOGETHER WITH the danger state is 71% against 23% - ~3.1x. So the caption under every dial quotes the measured risk of the band the needle is actually in rather than a generic legend, and says the weak/strong distinction in words. A unit test pins P(red AND danger) &gt; P(red) so the exhibit can never be re-worded into implying the needle is sufficient on its own. Every percentage printed is read from gauge_zones.json; a test greps the function body to prove neither edge is a literal in dashboard.py, and with the JSON absent the dial DECLINES TO EXIST rather than inventing bands.</t>
         </is>
       </c>
-      <c r="D22" s="33" t="inlineStr">
+      <c r="D22" s="35" t="inlineStr">
         <is>
           <t>all figures live in docs/research/gauge_zones.json</t>
         </is>
       </c>
-      <c r="E22" s="33" t="inlineStr">
+      <c r="E22" s="35" t="inlineStr">
         <is>
           <t>MEASURED - written by notebook 06's own code</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="32" t="inlineStr">
+      <c r="A23" s="34" t="inlineStr">
         <is>
           <t>GAUGE - STATE, never an instruction</t>
         </is>
       </c>
-      <c r="B23" s="33" t="inlineStr">
+      <c r="B23" s="35" t="inlineStr">
         <is>
           <t>gauge_state returns descriptive labels only: 'calm', 'warming', 'RED ZONE', 'RED ZONE + already run up'. A caption beside every dial states that GET IN and GET OUT come from the walk-forward detector and can fire with the needle anywhere.</t>
         </is>
       </c>
-      <c r="C23" s="33" t="inlineStr">
+      <c r="C23" s="35" t="inlineStr">
         <is>
           <t>A dial next to a trade signal will be read as a trade signal unless it is explicitly fenced. A unit test asserts the words 'get in' and 'get out' can never appear in a band label, at any level, in or out of the danger state.</t>
         </is>
       </c>
-      <c r="D23" s="33" t="inlineStr">
+      <c r="D23" s="35" t="inlineStr">
         <is>
           <t>n/a - invariant</t>
         </is>
       </c>
-      <c r="E23" s="33" t="inlineStr">
+      <c r="E23" s="35" t="inlineStr">
         <is>
           <t>INVARIANT - unit-tested</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="32" t="inlineStr">
+      <c r="A24" s="34" t="inlineStr">
         <is>
           <t>GAUGE - two layout defects found only by RENDERING and LOOKING</t>
         </is>
       </c>
-      <c r="B24" s="33" t="inlineStr">
+      <c r="B24" s="35" t="inlineStr">
         <is>
           <t>(i) plotly draws an Indicator `title` inside the SAME domain as the arc, so the two-line header was struck through by the navy value bar; the header is now paper-space annotations in the top margin. (ii) The value bar was thinned from thickness 0.28 to 0.15.</t>
         </is>
       </c>
-      <c r="C24" s="33" t="inlineStr">
+      <c r="C24" s="35" t="inlineStr">
         <is>
           <t>The desk has twice previously rejected charts for label-collision defects, and this project's own standard for the dial is that it and the curve beneath it 'can never disagree' - an illegible dial disagrees with everything. The bar thinning matters for the same reason: at 0.28 the navy sweep covered the very band colours it is supposed to be read against, so the red zone stopped being visible at exactly the moment it mattered. Both were invisible in code review and obvious in a rendered PNG.</t>
         </is>
       </c>
-      <c r="D24" s="33" t="inlineStr">
+      <c r="D24" s="35" t="inlineStr">
         <is>
           <t>height 268, margin t=64/b=36, bar thickness 0.15</t>
         </is>
       </c>
-      <c r="E24" s="33" t="inlineStr">
+      <c r="E24" s="35" t="inlineStr">
         <is>
           <t>FIXED - re-rendered and visually re-checked</t>
         </is>
       </c>
     </row>
     <row r="25" s="13">
-      <c r="A25" s="32" t="inlineStr">
+      <c r="A25" s="34" t="inlineStr">
         <is>
           <t>Feature bank HAND-SPECIFIED, not searched</t>
         </is>
       </c>
-      <c r="B25" s="33" t="inlineStr">
+      <c r="B25" s="35" t="inlineStr">
         <is>
           <t>The five onset features (attention_accel, hype_ratio, bull_inflection, influx_speed, attention_convexity) were each specified by hand, and every window inside them is a constant already validated elsewhere in the project: ROLL=7, the A1 120d hype baseline, the fade rule's 14d, E5's 60d LPPLS window. No stepwise selection, no L1 path, no genetic/automated search over the daily aggregates was used.</t>
         </is>
       </c>
-      <c r="C25" s="33" t="inlineStr">
+      <c r="C25" s="35" t="inlineStr">
         <is>
           <t>CONSIDERED AND REFUSED, and the reason is the SAMPLE, not a taste for handwork. The plausibly-independent unit of evidence here is the INSTRUMENT - 59 of them - not the day; the daily rows inside one name are one episode seen 4,000 times. A search that scores candidates against 183k daily rows is therefore choosing among thousands of options on an effective n of 59, which is exactly the regime where selection noise dominates and the in-sample winner does not survive walk-forward. Because every window is inherited, no feature adds a degree of freedom that a test year has not already seen. THE COST IS STATED OPENLY rather than hidden: per-feature AUROCs are only 0.51-0.60, and a search would very likely have posted better IN-SAMPLE numbers - that is the trade, made deliberately, and it is the same trade [1] sec 6.2.3 makes.</t>
         </is>
       </c>
-      <c r="D25" s="33" t="inlineStr">
+      <c r="D25" s="35" t="inlineStr">
         <is>
           <t>n/a - a methodology choice, not a fitted number</t>
         </is>
       </c>
-      <c r="E25" s="33" t="inlineStr">
+      <c r="E25" s="35" t="inlineStr">
         <is>
           <t>RECORDED 2026-07-27 (the decision itself dates from 2026-07-24; it had only ever been implicit, and the audit found it was recorded nowhere)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="32" t="inlineStr">
+      <c r="A26" s="34" t="inlineStr">
         <is>
           <t>THREE euphoria stores kept - none is a loser to delete</t>
         </is>
       </c>
-      <c r="B26" s="33" t="inlineStr">
+      <c r="B26" s="35" t="inlineStr">
         <is>
           <t>euphoria_desk.parquet + euphoria_desk_report.json = THE HEADLINE GET IN / GET OUT the euphoria tabs draw (dashboard.py:1732). euphoria_onset.parquet = the documented FALLBACK used only when the desk store is absent (dashboard.py:1750). euphoria_report.json = the FROZEN WALK-FORWARD thresholds, and the source of the gauge's red edge = 85 (dashboard.py:1887) plus the scorecard fallback (dashboard.py:2211).</t>
         </is>
       </c>
-      <c r="C26" s="33" t="inlineStr">
+      <c r="C26" s="35" t="inlineStr">
         <is>
           <t>The audit question was 'which report does the dashboard treat as headline, and remove the loser'. The answer is that there is no loser: the three stores do three different jobs and each is load-bearing. Removing the onset store would turn a graceful degradation into a crash on a fresh clone. Removing euphoria_report.json would be worse - it would turn the gauge's red edge from a number READ BACK OUT of the walk-forward into a hard-coded 85, i.e. it would manufacture exactly the arbitrary threshold the whole project exists to avoid. Recorded so the question is not re-opened at a defence.</t>
         </is>
       </c>
-      <c r="D26" s="33" t="inlineStr">
+      <c r="D26" s="35" t="inlineStr">
         <is>
           <t>GET IN 0.8481409001956947 / GET OUT 0.6302309197651663 (desk report); red edge 85 (walk-forward, every test year 2018-2026)</t>
         </is>
       </c>
-      <c r="E26" s="33" t="inlineStr">
+      <c r="E26" s="35" t="inlineStr">
         <is>
           <t>RESOLVED 2026-07-27 - nothing removed, and now documented</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="32" t="inlineStr">
+      <c r="A27" s="34" t="inlineStr">
         <is>
           <t>notebooks/PROJECT_SUMMARY.md DELETED</t>
         </is>
       </c>
-      <c r="B27" s="33" t="inlineStr">
+      <c r="B27" s="35" t="inlineStr">
         <is>
           <t>A 28KB unreferenced 'complete project guide' / reading-guide, last coherent before the 2026-07-24 desk pivot. Referenced by no code, no doc, no test.</t>
         </is>
       </c>
-      <c r="C27" s="33" t="inlineStr">
+      <c r="C27" s="35" t="inlineStr">
         <is>
           <t>DELETED BECAUSE IT HAD BECOME A CONTRADICTION SOURCE against the research report inside the same repo - the single most dangerous artefact to leave lying around before a defence. 19 of its headline numbers were stale or outright wrong: episodes 211 vs the true 333; data period 2021-2026 vs 2017-2026; onset capture 66% vs the measured 23.2%; top capture 68% vs the measured 13.1%; false alarms '0.23 budget maintained' vs the measured 0.348, i.e. 50% OVER budget, which the report lists as Limitation 4 'not hidden, not excused'; lead time '17 days BEFORE episode starts' vs the measured 17 days AFTER the trough - SIGN-FLIPPED; onset AP 0.0062 vs 0.098, off by ~16x; test years '2025-2026 only' vs 2018-2026; alert precision '~75%' vs the measured 0.21 START / 0.34 END; START edge '+2-5% vs baseline' vs the measured -0.81% at 21d with a CI containing zero. It also INVENTED a ground-truth rule that exists nowhere in the code ('G3 duration &gt;= 10 calendar days') and preserved a FALSE record of why phase-aware gating was rejected ('requires cheating') when the real recorded reason is measured and different. THREE UNIQUE ITEMS WERE MIGRATED BEFORE DELETION so no learning was lost: (i) the hand-specified-vs-searched rejection -&gt; the row above + RESEARCH_REPORT sec 5.2; (ii) the bootstrap replication count -&gt; PARAMETER_REGISTER Class 3; (iii) three primary citations (Hanley &amp; McNeil 1982, van Rijsbergen 1979, Matthews 1975) -&gt; References 15-17. Two further unique items were deliberately NOT migrated: its asset-class scope caveat (contradicted by the commodities-in-universe decision) and its crowd-lag rationale for the 7d windows (unmeasured assertion). Side benefit: it was the ONLY file in the repo carrying true emoji (15 codepoints) plus a U+FFFD corruption, so its removal closes the 'remove emojis' task.</t>
         </is>
       </c>
-      <c r="D27" s="33" t="inlineStr">
+      <c r="D27" s="35" t="inlineStr">
         <is>
           <t>n/a - a document, no parameters</t>
         </is>
       </c>
-      <c r="E27" s="33" t="inlineStr">
+      <c r="E27" s="35" t="inlineStr">
         <is>
           <t>DELETED 2026-07-27 after a line-by-line uniqueness audit against RESEARCH_REPORT / PARAMETER_REGISTER / ARCHITECTURE / README</t>
         </is>
       </c>
     </row>
     <row r="28" s="13">
-      <c r="A28" s="32" t="inlineStr">
+      <c r="A28" s="34" t="inlineStr">
         <is>
           <t>EUPHORIA PANEL quotes the threshold that actually FIRED (2026-07-28)</t>
         </is>
       </c>
-      <c r="B28" s="33" t="inlineStr">
+      <c r="B28" s="35" t="inlineStr">
         <is>
           <t>The lower panel now draws the frozen DESK threshold that gated the flags on screen (GET OUT 0.6302 / GET IN 0.8481, x100 onto the panel's existing 0-100 axis) and overlays the desk SCORE that crossed it, as lines+markers with connectgaps=False. Only alert kinds that actually fired inside the window are drawn. The level-detector's 85 line survives ONLY on the no-desk-store fallback path, where the level really is the decider.</t>
         </is>
       </c>
-      <c r="C28" s="33" t="inlineStr">
+      <c r="C28" s="35" t="inlineStr">
         <is>
           <t>BUG FIX, and the desk's complaint was a correct reading of a WRONG CHART. Verbatim: 'its quite unclear to see WHEN is the actual change / or get out flag - i want it to be like a clear peak or something (as right now its like flat and then suddently a get out flag)'. The old panel drew ONE dotted line at the level-detector's walk-forward threshold (85) and plotted the euphoria LEVEL against it - but when the desk store is present, which is the normal case, the flags are produced by the desk score crossing its OWN threshold. MEASURED over all 95 GET OUT alerts in the store: the plotted level was BELOW the drawn 85 line on 79 of them (83%), median plotted level at a GET OUT 74.8. So the chart showed a curve sitting comfortably under the line it said mattered, and then a flag appeared anyway. Nothing about the signal changed; the chart stopped contradicting it. The score is drawn sparse-by-construction (out_score exists on 2.5% of name-days, in runs as short as one day) because the gaps are information: no score means 'not judgeable here'.</t>
         </is>
       </c>
-      <c r="D28" s="33" t="inlineStr">
+      <c r="D28" s="35" t="inlineStr">
         <is>
           <t>No new number. GET OUT 0.6302309197651663 / GET IN 0.8481409001956947 read from euphoria_desk_report.json; x100 for the shared axis</t>
         </is>
       </c>
-      <c r="E28" s="33" t="inlineStr">
+      <c r="E28" s="35" t="inlineStr">
         <is>
           <t>SHIPPED 2026-07-28 - PARAMETER_REGISTER Class 8</t>
         </is>
       </c>
     </row>
     <row r="29" s="13">
-      <c r="A29" s="32" t="inlineStr">
+      <c r="A29" s="34" t="inlineStr">
         <is>
           <t>PEAK MARKER on the euphoria curve (2026-07-28)</t>
         </is>
       </c>
-      <c r="B29" s="33" t="inlineStr">
+      <c r="B29" s="35" t="inlineStr">
         <is>
           <t>The window maximum of the 7d-smoothed display curve is marked with a dot and a dated label ('peak 99 - 27 Jun'), with the value and full date in the hover. Passed to plotly as pd.DatetimeIndex([d]), not as a bare [Timestamp].</t>
         </is>
       </c>
-      <c r="C29" s="33" t="inlineStr">
+      <c r="C29" s="35" t="inlineStr">
         <is>
           <t>DESK REQUEST, verbatim: 'i want it to be like a clear peak or something'. It is a LABEL on a value already plotted, not a new quantity and not a threshold - nothing about the signal changes if it is removed, which is the test for whether a display addition is safe. The DatetimeIndex detail is a real defect avoided rather than a style note: a bare Timestamp inside a Python list survives the live app (streamlit serialises through plotly's own encoder) but is NOT JSON-serialisable by kaleido, so a one-element list silently breaks static PNG export - and these panels are exported for the LaTeX decks.</t>
         </is>
       </c>
-      <c r="D29" s="33" t="inlineStr">
+      <c r="D29" s="35" t="inlineStr">
         <is>
           <t>n/a - a label on the plotted curve</t>
         </is>
       </c>
-      <c r="E29" s="33" t="inlineStr">
+      <c r="E29" s="35" t="inlineStr">
         <is>
           <t>SHIPPED 2026-07-28</t>
         </is>
       </c>
     </row>
     <row r="30" s="13">
-      <c r="A30" s="32" t="inlineStr">
+      <c r="A30" s="34" t="inlineStr">
         <is>
           <t>GAUGE answers 'now' AND 'this window' (2026-07-28)</t>
         </is>
       </c>
-      <c r="B30" s="33" t="inlineStr">
+      <c r="B30" s="35" t="inlineStr">
         <is>
           <t>The big needle still reads TODAY (the last day of the selected window). Added behind it: the window's high-water mark as one dated line - 'window high 99 (RED ZONE) on 27 Jun', or 'this IS the window's high point' when the two are within 1 point. Drawn as TEXT, not a second needle. Frame grows 268 -&gt; 300px, bottom margin 36 -&gt; 74px. Separately, the standing explanation moved off the page into the info hover (help=), leaving one headline line beside each dial.</t>
         </is>
       </c>
-      <c r="C30" s="33" t="inlineStr">
+      <c r="C30" s="35" t="inlineStr">
         <is>
           <t>BUG FIX BY EXPLANATION - no edge moved and no number was invented. Desk report: 'the gauge, it seems to alwahys show calm'. The dial was not stuck. MEASURED over the default window (2026-01-01 -&gt; latest): 50 of 59 instruments read calm at the last day while 17 of those SAME names touched the RED ZONE somewhere inside the window. Both are true at once because the page is ordered by MOST RECENT SIGNAL, so a name earns its place with an episode that may have peaked months ago while the needle - correctly - reports today. A dial that answers 'how hot is it now?' on a name selected for 'it was hot recently' reads calm almost always and looks broken while being right. Softening an edge to make it look busier would have been exactly the arbitrary-threshold move this project refuses; making the dial answer both questions costs nothing and is honest. TEXT rather than a second needle because plotly's Indicator has a single threshold slot and it already carries the red edge as a hard line (colour alone does not survive greyscale or a projector); faking a second needle means drawing shapes against the arc's internal geometry in paper space, fragile across plotly versions, and two needles on a 268px dial reads worse than one sentence. The hover move is the desk's own instruction ('dont need to explain it fully all the time, maybe an info icon hover or something'): the dial used to print a measured-percentage paragraph plus a four-sentence caption on EVERY chart, so a page of six names carried the same ~90 words six times. The evidence is not deleted or weakened - it is one hover away, available when someone challenges the band and silent when nobody is asking.</t>
         </is>
       </c>
-      <c r="D30" s="33" t="inlineStr">
+      <c r="D30" s="35" t="inlineStr">
         <is>
           <t>No edge changed: red 85, amber 76. Display only: valueformat '.0f' on number and delta (a tenth of a percentile-rank index is below the resolution of the input)</t>
         </is>
       </c>
-      <c r="E30" s="33" t="inlineStr">
+      <c r="E30" s="35" t="inlineStr">
         <is>
           <t>SHIPPED 2026-07-28 - PARAMETER_REGISTER Class 8</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="34" t="inlineStr">
+        <is>
+          <t>ONE READINESS LINE replaces the five-overlay euphoria panel (2026-07-28)</t>
+        </is>
+      </c>
+      <c r="B31" s="35" t="inlineStr">
+        <is>
+          <t>The panel now draws one series per firing rule: readiness = deciding score / that rule's frozen threshold x 100. The firing line is therefore ALWAYS 100, for every name, every rule, every window. Both rules share one dotted line. Near-misses are drawn too (any rule whose score exists in the window), and gaps stay gaps (connectgaps=False). The raw level, the smoothed level, the eligibility ribbon and the second threshold line are off the panel; the level now lives on the dial above it.</t>
+        </is>
+      </c>
+      <c r="C31" s="35" t="inlineStr">
+        <is>
+          <t>DISPLAY DERIVATION - no new quantity, no number moved. Desk report: 'the euphoria charts are still way too messy. i dont get what is activating a signal, is it a crossing? inflection? i just want one line'. It IS a crossing - alerts_from_scores fires on score &gt;= threshold with a 21-day cooldown, and there is no inflection test anywhere in the firing path - but the old panel could not show that: five elements at equal weight, and the two thresholds (GET IN 0.848141, GET OUT 0.630231) at DIFFERENT heights, so neither line meant 'the line'. Dividing each score by its own threshold is what lets one line mean it. Near-misses are drawn because with the level gone, a name that never alerted would otherwise show an empty panel - and a line that climbs to 80 and turns over IS the answer to 'why did nothing fire here?'.</t>
+        </is>
+      </c>
+      <c r="D31" s="35" t="inlineStr">
+        <is>
+          <t>Same stored scores, same frozen thresholds (0.630231 / 0.848141), divided. ALERT DATES ARE BIT-IDENTICAL; the vertical signal lines still come from `coherent`. Measured sparsity, since it is visible on screen: over 63,345 name-days the deciding score exists on 2.5% of days for GET OUT and 48.8% for GET IN; the 1,600 GET OUT scored days form 160 runs of MEDIAN LENGTH 7 DAYS (mean 10, max 91, only 28 single days).</t>
+        </is>
+      </c>
+      <c r="E31" s="35" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-07-28 - PARAMETER_REGISTER Class 8 (continued)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="34" t="inlineStr">
+        <is>
+          <t>PERFORMANCE METRICS REMOVED from the dashboard (2026-07-28)</t>
+        </is>
+      </c>
+      <c r="B32" s="35" t="inlineStr">
+        <is>
+          <t>No hit rate, lead time, false-alarm count or confidence interval appears anywhere on the dashboard. All performance reporting lives in the notebooks, notebook 07 in particular.</t>
+        </is>
+      </c>
+      <c r="C32" s="35" t="inlineStr">
+        <is>
+          <t>DESK DECISION. 'remove the hit rate etc stuff (the perfomance metrics) in the dashboard i will just keep this for the notebooks only.' Consistent with the standing split: the notebooks are the research record, the dashboard states conclusions only.</t>
+        </is>
+      </c>
+      <c r="D32" s="35" t="inlineStr">
+        <is>
+          <t>SCOPE, stated so it can be challenged: headline performance reporting is gone everywhere, but the justification numbers inside decisions_simple() / DECISIONS_DOC and the band-meaning percentages in gauge_caption() were KEPT. Removing those would leave every remaining choice on the page looking arbitrary, which is the failure mode the parameter register exists to prevent. Alex can override.</t>
+        </is>
+      </c>
+      <c r="E32" s="35" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-07-28 - PARAMETER_REGISTER Class 8 (continued)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="34" t="inlineStr">
+        <is>
+          <t>PANEL LAYOUT: header, then dial + facts on ONE row, then the chart (2026-07-28)</t>
+        </is>
+      </c>
+      <c r="B33" s="35" t="inlineStr">
+        <is>
+          <t>The instrument name is a single compact header line with its symbol and state badge. The dial shares one row with five facts: state, today's reading, the 7-day change, the window peak, the last signal. The figure follows immediately with title=None and an 8px top margin.</t>
+        </is>
+      </c>
+      <c r="C33" s="35" t="inlineStr">
+        <is>
+          <t>DESK DECISION. 'arrange the dashboard better / like title of ticker / guage + some elements next to it / then chart / essentially using less white space'. The old stack paid for a half-used dial row plus a second title strip inside the figure's own 55px top margin - per name, which on a six-name page is most of a screen spent on furniture.</t>
+        </is>
+      </c>
+      <c r="D33" s="35" t="inlineStr">
+        <is>
+          <t>The five facts all answer WHERE THIS NAME IS. None answers how well the detector has done - that is the no-performance-metrics decision above, honoured in the one place where there was now room to break it.</t>
+        </is>
+      </c>
+      <c r="E33" s="35" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-07-28 - PARAMETER_REGISTER Class 8 (continued)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="34" t="inlineStr">
+        <is>
+          <t>PLAIN-ENGLISH OPENER KEPT ('what is euphoria - start here') (2026-07-28)</t>
+        </is>
+      </c>
+      <c r="B34" s="35" t="inlineStr">
+        <is>
+          <t>The plain-English explainer at the top of the dashboard stays.</t>
+        </is>
+      </c>
+      <c r="C34" s="35" t="inlineStr">
+        <is>
+          <t>DESK DECISION, explicitly retained: 'keep the what is euphoria- start here - plan english on the dasboard, i like it'. Recorded because it was kept during a pass whose whole direction was removal.</t>
+        </is>
+      </c>
+      <c r="D34" s="35" t="inlineStr">
+        <is>
+          <t>None. Prose only.</t>
+        </is>
+      </c>
+      <c r="E34" s="35" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-07-28 - kept on instruction</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="34" t="inlineStr">
+        <is>
+          <t>GET IN lead time reported on TWO CLOCKS (2026-07-28)</t>
+        </is>
+      </c>
+      <c r="B35" s="35" t="inlineStr">
+        <is>
+          <t>Notebook 07's final scorecard carries two separate rows: 'days from alert to the peak' and 'days from the trough to the alert'. For GET OUT the first IS the warning and the second is n/a. For GET IN the first is the rally still ahead (69 days) and the second is the entry lag (16.5 days).</t>
+        </is>
+      </c>
+      <c r="C35" s="35" t="inlineStr">
+        <is>
+          <t>CORRECTION of a reporting defect introduced by the scorecard itself. A single 'median warning' row collapsed two different clocks into one label, and for a START signal it printed 69 days - arithmetically correct, editorially wrong, and in direct contradiction with the shipped record (16) and the deck (17 after the trough / 66 ahead). A PM comparing the two would have been right to distrust both.</t>
+        </is>
+      </c>
+      <c r="D35" s="35" t="inlineStr">
+        <is>
+          <t>No detector change. The saved final_verdict['get_in']['median_lead_d'] now uses the after-trough clock (the shipped record's convention) with median_rally_ahead_d carrying the other. 16.5 here vs 16 in the record is the SAME statistic: euphoria_phases.py truncates with int(np.median(...)).</t>
+        </is>
+      </c>
+      <c r="E35" s="35" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-07-28 - notebook 07 PART D</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="34" t="inlineStr">
+        <is>
+          <t>SHORT DECK rewritten as an adoption case, v1.1 (2026-07-28)</t>
+        </is>
+      </c>
+      <c r="B36" s="35" t="inlineStr">
+        <is>
+          <t>docs/presentation/retailradar_short.tex rewritten end to end. Every slide leads with what the desk gets and closes with the evidence for it. The three negative-result slides stay, reframed as the warrant for the positive ones rather than as a hedge. Closes with an explicit ask: run it live on the book for a quarter.</t>
+        </is>
+      </c>
+      <c r="C36" s="35" t="inlineStr">
+        <is>
+          <t>DESK DECISION. 'change the tone of hte presentation files (the tex) to be like more positive towards the project... i need to sell this project to my boss to adopt'. Scope was confirmed with Alex as the 15-slide short deck ONLY; retailradar_presentation.tex is deliberately untouched.</t>
+        </is>
+      </c>
+      <c r="D36" s="35" t="inlineStr">
+        <is>
+          <t>NOT ONE FIGURE WAS CHANGED to achieve the tone - every number in the deck is the number the notebooks print. That fact is stated in the .tex header block so it survives a challenge. Build verified: 15 pages, 0 overfull vbox, 0 errors, against a pre-edit baseline built in the same directory to prove the rewrite cost nothing typographically.</t>
+        </is>
+      </c>
+      <c r="E36" s="35" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-07-28 - deck version 'short v1.1'</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="34" t="inlineStr">
+        <is>
+          <t>FIRING PATH written out end to end (2026-07-28)</t>
+        </is>
+      </c>
+      <c r="B37" s="35" t="inlineStr">
+        <is>
+          <t>The GET IN / GET OUT mechanism specified as ONE path in RESEARCH_REPORT 6.14: (1) candidacy - GET OUT needs hype_ok AND boom_state, GET IN needs hype_raw &gt;= 1 AND NOT end_stage_mask; (2) score - unweighted mean of the bank (GET OUT e1,e2,e3,e5,fade with the A2/A3 gates re-expressed in score space; GET IN attention_accel,hype_ratio,bull_inflection,influx_speed,attention_convexity), no fitting because the family is rules; (3) trailing 7-day per-name mean, no look-ahead; (4) np.flatnonzero(score &gt;= threshold) then a 21-day cooldown then the asymmetric coherence machine.</t>
+        </is>
+      </c>
+      <c r="C37" s="35" t="inlineStr">
+        <is>
+          <t>The desk asked 'how does it actually work? the signal for get in / get out?' AFTER the panel rebuild claimed to answer it. The mechanism existed in shipped source but was distributed across report 6.7, 6.8, a register class and four files, so nobody could trace it in one read. A detector that cannot be traced end to end cannot be defended in a room. IT IS A CROSSING: there is no inflection, peak or convexity test anywhere in the firing path - the convexity in the GET IN bank is a feature being averaged, not a trigger. Price inside the GET OUT gate is ELIGIBILITY ONLY, never a scored feature.</t>
+        </is>
+      </c>
+      <c r="D37" s="35" t="inlineStr">
+        <is>
+          <t>No parameter changed. Documentation only. Frozen thresholds restated: GET OUT 0.630231, GET IN 0.848141, ROLL=7, EUPHORIA_COOLDOWN_DAYS=21.</t>
+        </is>
+      </c>
+      <c r="E37" s="35" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-07-28 - report 6.14, register Class 8 third pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="34" t="inlineStr">
+        <is>
+          <t>STREAMLIT TITLE BUG - title must be an explicit EMPTY STRING (2026-07-28)</t>
+        </is>
+      </c>
+      <c r="B38" s="35" t="inlineStr">
+        <is>
+          <t>dashboard.py draw_chart sets title=dict(text="") on the euphoria figure instead of leaving the title unset.</t>
+        </is>
+      </c>
+      <c r="C38" s="35" t="inlineStr">
+        <is>
+          <t>BUG FIX, root-caused in the live DOM. A bold 'undefined' was printing over every euphoria chart and the word appears in NO Python file in this repo; four source-level hypotheses were formed and discarded before the DOM was dumped. Walking the tspan's ancestor chain and reading data-unformatted on text.gtitle returned '&lt;b&gt;&lt;b&gt;undefined&lt;/b&gt;&lt;/b&gt;', which named the layer and the mechanism: Streamlit's plotly theming rewrites the title as '&lt;b&gt;' + spec.layout.title.text + '&lt;/b&gt;', and with the title strip deliberately absent (it cost 55px of dead space per name) that inner value is the JavaScript undefined. An empty string is a real string, so the same rewrite yields '&lt;b&gt;&lt;/b&gt;' and renders nothing. Lesson repeated from the 2026-07-27 influence re-cut: when the source does not contain the symptom, the rendered object does.</t>
+        </is>
+      </c>
+      <c r="D38" s="35" t="inlineStr">
+        <is>
+          <t>Display only. Verified live: rendered _fullLayout.title.text = '&lt;b&gt;&lt;b&gt;&lt;/b&gt;&lt;/b&gt;'; occurrences of 'undefined' on the page 6 -&gt; 0.</t>
+        </is>
+      </c>
+      <c r="E38" s="35" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-07-28 - verified in the browser</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="34" t="inlineStr">
+        <is>
+          <t>TOP MARGIN 8px -&gt; 38px, derived from the label geometry (2026-07-28)</t>
+        </is>
+      </c>
+      <c r="B39" s="35" t="inlineStr">
+        <is>
+          <t>The euphoria figure's top margin is 38px.</t>
+        </is>
+      </c>
+      <c r="C39" s="35" t="inlineStr">
+        <is>
+          <t>BUG FIX. The 'GET OUT &lt;date&gt;' labels were being cut in half by the canvas edge. DERIVED, not tuned: the annotations sit at y=1.0, yref='y domain', yanchor='bottom' with alternating yshift = 4 + 14*(i%2) (so up to 18) to stop adjacent labels colliding, and 9.5px text is about 13px tall, so the tallest label reaches roughly 31px ABOVE the price panel. 38 clears 31 with a little air and is still LESS than the 55px the deleted title strip cost, so the space saving that motivated removing the title survives.</t>
+        </is>
+      </c>
+      <c r="D39" s="35" t="inlineStr">
+        <is>
+          <t>margin.t = 38 (was 8). Display only; verified live.</t>
+        </is>
+      </c>
+      <c r="E39" s="35" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-07-28 - all four labels legible in the screenshot</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="34" t="inlineStr">
+        <is>
+          <t>THE GHOST LINE - a knowing reversal, made safe by three guards (2026-07-28)</t>
+        </is>
+      </c>
+      <c r="B40" s="35" t="inlineStr">
+        <is>
+          <t>Each readiness series is drawn a SECOND time underneath the measured trace: the same values time-interpolated across gaps, 1px, dotted, 30% opacity, excluded from the legend, added first so it renders behind.</t>
+        </is>
+      </c>
+      <c r="C40" s="35" t="inlineStr">
+        <is>
+          <t>DESK DECISION: 'can we make the euphoria still have like a continuos line? but maybe make it like not as prominant'. The arcs are correct but leave the eye nothing to follow, so a reader has to reconstruct the episode shape themselves. THIS REVERSES the same-day rejection of a dense line (rejected because it 'invents a reading on ungated days'), so it is only defensible with the reason the old version was unsafe identified and removed. (1) hoverinfo='skip' - the ghost NEVER reports a number; hover still comes only from the bold trace, so no ungated day can be read off the screen as a score. This is the load-bearing guard: the earlier objection was to a dense line that could be QUERIED, not one that could be SEEN. (2) limit_area='inside' - interpolation happens only BETWEEN two real scored days, never past the first or last, so the ghost cannot imply a reading in a stretch the detector never judged at all. (3) 1px dotted at 30% with no legend entry - it reads as a construction line; the solid 2.4px markered trace is still the only thing on the panel that looks like a measurement. The lower-panel caption states all of this in plain English, because a faint line that cannot be hovered is only honest if the panel says so.</t>
+        </is>
+      </c>
+      <c r="D40" s="35" t="inlineStr">
+        <is>
+          <t>NOTHING FEEDS THE MODEL. Alert dates bit-identical. Verified live: two '(shape only)' traces with hoverinfo='skip', connectgaps=true, opacity=0.3.</t>
+        </is>
+      </c>
+      <c r="E40" s="35" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-07-28 - verified in the browser</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="34" t="inlineStr">
+        <is>
+          <t>FOUR EXPLANATION EXPANDERS REMOVED from the dashboard (2026-07-28)</t>
+        </is>
+      </c>
+      <c r="B41" s="35" t="inlineStr">
+        <is>
+          <t>Removed: page-level 'WHY THE MODEL DOES WHAT IT DOES' (decisions_simple(), 7 decisions each with the number that settled it) and the long-form evidence log (DECISIONS_DOC); euphoria-tab 'full method &amp; measured record' (EUPHORIA_DEF_FULL) and the deep archive that read docs/PARAMETER_REGISTER.md off disk and printed the whole file. ONE explainer survives and its label is FROZEN VERBATIM: 'what is euphoria?  (start here - plain English)'.</t>
+        </is>
+      </c>
+      <c r="C41" s="35" t="inlineStr">
+        <is>
+          <t>DESK DECISION: 'for the explanations, just keep the what is euphoria one ... dont change the current what is euphoria? (start here - plain English) just remove the rest'. A proposed rename to 'What is Euphoria' was withdrawn in the same exchange and that withdrawal is recorded so it is not re-litigated. Consistent with the standing split: the notebooks and the register are the research record, the terminal states conclusions - and all four expanders were second copies of DECISIONS.xlsx, PARAMETER_REGISTER.md and the notebooks, so no reasoning is lost. WHAT IT COSTS, recorded because the argument went the other way and was overruled: a PM who challenges a threshold live can no longer answer it from this page; the answer now requires the register or a notebook.</t>
+        </is>
+      </c>
+      <c r="D41" s="35" t="inlineStr">
+        <is>
+          <t>decisions_simple(), DECISIONS_DOC and EUPHORIA_DEF_FULL are left DEFINED BUT UNREFERENCED rather than deleted, so restoring any of this is a two-line change. THEY ARE EXEMPT FROM THE NO-DEAD-CODE SWEEP.</t>
+        </is>
+      </c>
+      <c r="E41" s="35" t="inlineStr">
+        <is>
+          <t>SHIPPED 2026-07-28 - four labels confirmed absent from the rendered page</t>
         </is>
       </c>
     </row>
@@ -4078,7 +5109,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4446,7 +5477,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4779,7 +5810,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4910,427 +5941,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" style="13" min="1" max="1"/>
-    <col width="52" customWidth="1" style="13" min="2" max="2"/>
-    <col width="46" customWidth="1" style="13" min="3" max="3"/>
-    <col width="40" customWidth="1" style="13" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="27" t="inlineStr">
-        <is>
-          <t>7b. Euphoria START detection - the July-2026 phases study (notebooks 01-04)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="28" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B3" s="28" t="inlineStr">
-        <is>
-          <t>Decision / result</t>
-        </is>
-      </c>
-      <c r="C3" s="28" t="inlineStr">
-        <is>
-          <t>Derivation (no arbitrary numbers)</t>
-        </is>
-      </c>
-      <c r="D3" s="28" t="inlineStr">
-        <is>
-          <t>Evidence</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="29" t="inlineStr">
-        <is>
-          <t>Aim</t>
-        </is>
-      </c>
-      <c r="B4" s="29" t="inlineStr">
-        <is>
-          <t>Detect the START of GME-scale euphoria episodes from the crowd alone, sparingly; plus confirm the TOP detector.</t>
-        </is>
-      </c>
-      <c r="C4" s="29" t="inlineStr">
-        <is>
-          <t>Extends the July-2026 re-aim; crowd-only hard rule unchanged (price = ground truth + scoring only).</t>
-        </is>
-      </c>
-      <c r="D4" s="29" t="inlineStr">
-        <is>
-          <t>notebooks/01-04; analytics/euphoria_phases.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="29" t="inlineStr">
-        <is>
-          <t>Episode ground truth</t>
-        </is>
-      </c>
-      <c r="B5" s="29" t="inlineStr">
-        <is>
-          <t>Boom-bust arc trough-&gt;peak-&gt;bust from the EXISTING peak rules G1-G3; trough = the 120d low G2 already measures the boom from.</t>
-        </is>
-      </c>
-      <c r="C5" s="29" t="inlineStr">
-        <is>
-          <t>No new fitted quantity: every threshold inherited from the validated top study.</t>
-        </is>
-      </c>
-      <c r="D5" s="29" t="inlineStr">
-        <is>
-          <t>NB01: 333 episodes, 126 onset-detectable, 136 top-detectable</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="29" t="inlineStr">
-        <is>
-          <t>Onset hit window</t>
-        </is>
-      </c>
-      <c r="B6" s="29" t="inlineStr">
-        <is>
-          <t>[trough, trough+45d], CAPPED at the peak; mid-rally alerts = LATE (neither hit nor false).</t>
-        </is>
-      </c>
-      <c r="C6" s="29" t="inlineStr">
-        <is>
-          <t>45d mirrors the existing FA horizon in score_alerts; cap prevents post-top alerts counting as 'caught the start'. Desk decision, recorded before results.</t>
-        </is>
-      </c>
-      <c r="D6" s="29" t="inlineStr">
-        <is>
-          <t>NB01 register; test_onset_window_capped_at_peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="29" t="inlineStr">
-        <is>
-          <t>Feature bank (locked)</t>
-        </is>
-      </c>
-      <c r="B7" s="29" t="inlineStr">
-        <is>
-          <t>attention_accel, hype_ratio, bull_inflection, influx_speed, attention_convexity.</t>
-        </is>
-      </c>
-      <c r="C7" s="29" t="inlineStr">
-        <is>
-          <t>Every window derived from existing constants (ROLL=7, 28d E-windows, 14d fade window, 120d hype baseline). source_breadth REJECTED: coverage-regime artifact (X/StockTwits exist only from 2026).</t>
-        </is>
-      </c>
-      <c r="D7" s="29" t="inlineStr">
-        <is>
-          <t>NB02 battery: per-feature AUROC + cluster-bootstrap CIs, ablation, perturbation</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="29" t="inlineStr">
-        <is>
-          <t>Tournament winner</t>
-        </is>
-      </c>
-      <c r="B8" s="29" t="inlineStr">
-        <is>
-          <t>RULES (unweighted bank mean, coverage + above-median-attention gates). GBM tied on AP but not outside the bootstrap CI -&gt; parsimony; MLP finished below random.</t>
-        </is>
-      </c>
-      <c r="C8" s="29" t="inlineStr">
-        <is>
-          <t>Criterion pre-stated: AP ranking (thesis 6.2.3), must beat random on AP+AUROC, parsimony CI rule; FA budget derived from the incumbent's accepted 0.23/instr-yr.</t>
-        </is>
-      </c>
-      <c r="D8" s="29" t="inlineStr">
-        <is>
-          <t>NB03: rules AP 0.098 vs random 0.072; top task: rules AP 0.286 vs random 0.204</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="29" t="inlineStr">
-        <is>
-          <t>Validated record</t>
-        </is>
-      </c>
-      <c r="B9" s="29" t="inlineStr">
-        <is>
-          <t>29/125 detectable onsets captured (23%), 21 late, 169 FA = 0.348/instr-yr (ABOVE the 0.23 budget - stated cost).</t>
-        </is>
-      </c>
-      <c r="C9" s="29" t="inlineStr">
-        <is>
-          <t>Walk-forward, thresholds from past years only; both denominators always reported.</t>
-        </is>
-      </c>
-      <c r="D9" s="29" t="inlineStr">
-        <is>
-          <t>NB04: median entry 17d after trough, 66d of rally still ahead</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="29" t="inlineStr">
-        <is>
-          <t>Label sensitivity</t>
-        </is>
-      </c>
-      <c r="B10" s="29" t="inlineStr">
-        <is>
-          <t>Capture rate flat across softened(20/40)/standard(25/50)/hardened(30/60) boom labels: 22.4%, 23.2%, 22.1%.</t>
-        </is>
-      </c>
-      <c r="C10" s="29" t="inlineStr">
-        <is>
-          <t>Thesis 7.1.2 port: conclusions must survive labelling perturbation.</t>
-        </is>
-      </c>
-      <c r="D10" s="29" t="inlineStr">
-        <is>
-          <t>NB03 sensitivity table</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="29" t="inlineStr">
-        <is>
-          <t>Trading translation</t>
-        </is>
-      </c>
-      <c r="B11" s="29" t="inlineStr">
-        <is>
-          <t>REJECTED for both ONSET-&gt;BUY and TOP-&gt;SELL under the pre-stated criterion (n&gt;=30, beats same-instrument 20d baseline, CI excludes 0).</t>
-        </is>
-      </c>
-      <c r="C11" s="29" t="inlineStr">
-        <is>
-          <t>Same treatment as the retired BUY/SELL engine; evidence retained.</t>
-        </is>
-      </c>
-      <c r="D11" s="29" t="inlineStr">
-        <is>
-          <t>NB04: onset diff -0.63% CI [-0.0151, 0.0026]; top diff -1.55% CI [-0.0563, 0.0263]</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="29" t="inlineStr">
-        <is>
-          <t>Dashboard</t>
-        </is>
-      </c>
-      <c r="B12" s="29" t="inlineStr">
-        <is>
-          <t>New 'Start / End radar' tab: STARTING and ENDING panes, each split Themes | Single names; only names alerted within the 21d cooldown; record printed on the pane.</t>
-        </is>
-      </c>
-      <c r="C12" s="29" t="inlineStr">
-        <is>
-          <t>Sparse by design - an empty pane is the radar working.</t>
-        </is>
-      </c>
-      <c r="D12" s="29" t="inlineStr">
-        <is>
-          <t>dashboard.py t_phase; AppTest 0 exceptions</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="29" t="inlineStr">
-        <is>
-          <t>Price-assisted END gate (2026-07-24)</t>
-        </is>
-      </c>
-      <c r="B13" s="29" t="inlineStr">
-        <is>
-          <t>PASSED all pre-stated conditions: G2 boom thresholds as a live prerequisite -&gt; capture 16-&gt;26 detectable tops (matched years), AP 0.286-&gt;0.435, FAs 44-&gt;41, capture-gain CI [+3.5pp,+13pp]. Offered as labelled second signal; claim becomes 'crowd + chart'.</t>
-        </is>
-      </c>
-      <c r="C13" s="29" t="inlineStr">
-        <is>
-          <t>The gate reuses the ground-truth boom definition on trailing prices - no new constant, no look-ahead.</t>
-        </is>
-      </c>
-      <c r="D13" s="29" t="inlineStr">
-        <is>
-          <t>NB03 commissioned-test section</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="29" t="inlineStr">
-        <is>
-          <t>Combined price+crowd ALERT bank (2026-07-24)</t>
-        </is>
-      </c>
-      <c r="B14" s="29" t="inlineStr">
-        <is>
-          <t>REJECTED under pre-stated criterion: 65% cliff-30 hit rate indistinguishable from its own 62% candidate-day baseline (CI includes 0). Smoothed-trigger evidence retained: FA 31-&gt;24 at equal capture, median trigger run 6-&gt;8d.</t>
-        </is>
-      </c>
-      <c r="C14" s="29" t="inlineStr">
-        <is>
-          <t>The alert layer cannot out-predict its own danger state; its job is timing the peak, which it does (median 8d lead).</t>
-        </is>
-      </c>
-      <c r="D14" s="29" t="inlineStr">
-        <is>
-          <t>NB06 desk-signal study</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="29" t="inlineStr">
-        <is>
-          <t>DANGER STATE shipped (2026-07-24)</t>
-        </is>
-      </c>
-      <c r="B15" s="29" t="inlineStr">
-        <is>
-          <t>The candidacy state (A1 2x hype AND G2 boom) validated as the standing drop-warning: cliff-30 = 62% in-state vs 19% ordinary, uplift CI [+28pp,+50pp]. Rendered as the amber band on every terminal price panel.</t>
-        </is>
-      </c>
-      <c r="C15" s="29" t="inlineStr">
-        <is>
-          <t>Pure composition of two existing constants; the single most actionable statistic of the project for the PM use case.</t>
-        </is>
-      </c>
-      <c r="D15" s="29" t="inlineStr">
-        <is>
-          <t>NB06; dashboard danger band; PARAMETER_REGISTER</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="29" t="inlineStr">
-        <is>
-          <t>DESK CONFIGURATION adopted: GET OUT (2026-07-24)</t>
-        </is>
-      </c>
-      <c r="B16" s="29" t="inlineStr">
-        <is>
-          <t>Boom-gated END rules + 7d-smoothed (ROLL) trigger. Walk-forward: capture 24/122 detectable tops, FA 39 (0.195/instr-yr), AP 0.449 (raw gate 0.435), median warning 8d before the peak. Smoothing adopted by pre-stated rule (AP not lower AND FAs not higher); 2-capture cost recorded. Frozen live threshold 0.630 (budget rule, full prior years).</t>
-        </is>
-      </c>
-      <c r="C16" s="29" t="inlineStr">
-        <is>
-          <t>The desk lifted the crowd-only rule for a labelled SECOND family ('use both price and social media - I want a better hit rate') and demanded no one-day blips. Candidacy = A1 hype AND G2 boom (existing constants only).</t>
-        </is>
-      </c>
-      <c r="D16" s="29" t="inlineStr">
-        <is>
-          <t>NB06 adopted-configuration section; euphoria_desk_report.json; euphoria_phases.py §6</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="29" t="inlineStr">
-        <is>
-          <t>DESK CONFIGURATION adopted: GET IN (2026-07-24)</t>
-        </is>
-      </c>
-      <c r="B17" s="29" t="inlineStr">
-        <is>
-          <t>Phase-aware onset (end-stage days - A1∧A2∧A3-persistence - excluded from candidacy) + 7d smoothing. Adjacency (START within 21d before an END) 20→2, LATE 21→10, FA 169→124; capture cost 29→20 of 125 RECORDED. Frozen live threshold 0.848. OVERRULES the earlier utility-rule rejection of the phase-aware variant as an explicit desk decision.</t>
-        </is>
-      </c>
-      <c r="C17" s="29" t="inlineStr">
-        <is>
-          <t>The desk stated three times that a START landing on an END destroys PM trust - adjacency is the binding constraint, so it overrules raw capture. Selection rule pre-stated in NB06; drift guard pins notebook == production.</t>
-        </is>
-      </c>
-      <c r="D17" s="29" t="inlineStr">
-        <is>
-          <t>NB06; euphoria_desk_report.json; PARAMETER_REGISTER class 5; dashboard GET IN/GET OUT banners</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="29" t="inlineStr">
-        <is>
-          <t>Improvement campaign: NOTHING adopted (2026-07-24, NB07)</t>
-        </is>
-      </c>
-      <c r="B18" s="29" t="inlineStr">
-        <is>
-          <t>Four pre-registered challengers vs the shipped desk configuration (adoption rule pre-stated: more captures, FAs not higher, paired cluster gain CI excluding zero): per-kind thresholds REJECTED (cap 23 vs 24 on unmatched years, though FA halved 39-&gt;16 - WATCH item); logistic-weighted score REJECTED by parsimony (30 vs 24 captures but gain CI [-1,+11] touches zero - WATCH item, auto re-test at year rollover); smoothing sweep w in {1,3,5,7,10,14}: no window dominates w=7; Western-Electric run rules k&gt;1: dominated by the smoothed single crossing.</t>
-        </is>
-      </c>
-      <c r="C18" s="29" t="inlineStr">
-        <is>
-          <t>The shipped configuration sits at the measured frontier. Watch items re-test automatically at the next --research pass under the same rule.</t>
-        </is>
-      </c>
-      <c r="D18" s="29" t="inlineStr">
-        <is>
-          <t>NB07 part B; nb07_performance_battery.json; RESEARCH_REPORT 6.9</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="29" t="inlineStr">
-        <is>
-          <t>Clustering-as-conviction REJECTED as exit criterion (2026-07-24, NB07)</t>
-        </is>
-      </c>
-      <c r="B19" s="29" t="inlineStr">
-        <is>
-          <t>The desk's 'buy-buy-buy / sell-sell-sell in a tight window' hypothesis, both forms: per-instrument intensity (trigger days in trailing 21d cooldown; STRONG = 2+ days) - cliff-30 rate 52.9% vs 55.9% single-day, uplift CI [-21pp,+22pp] straddles zero; cross-market breadth (share of names in GET OUT within 7d, top decile) - basket fwd-21d not separable at 90% (block bootstrap). A second GET OUT inside an episode is the same sell, not more sell.</t>
-        </is>
-      </c>
-      <c r="C19" s="29" t="inlineStr">
-        <is>
-          <t>The exit criterion remains the GET OUT alert itself; the cooldown + smoothed trigger already absorb repetition. The standing warning remains the danger-state band (NB06).</t>
-        </is>
-      </c>
-      <c r="D19" s="29" t="inlineStr">
-        <is>
-          <t>NB07 part C; RESEARCH_REPORT 6.9</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="29" t="inlineStr">
-        <is>
-          <t>Performance battery adopted into the research record (2026-07-24, NB07)</t>
-        </is>
-      </c>
-      <c r="B20" s="29" t="inlineStr">
-        <is>
-          <t>Literature-grounded metrics added: PR/F1/MCC at the operating point (Davis &amp; Goadrich; Chicco &amp; Jurman), delay-vs-FA frontier (Page 1954), MacKinlay CAR with cluster CIs, reliability diagram (Murphy &amp; Winkler), Grinold-Kahn IC, overlay Sharpe/Sortino (descriptive). The positive daily IC (+0.11) is recorded as PROOF the detector is an episode alarm, not daily alpha - a defense point, not a defect.</t>
-        </is>
-      </c>
-      <c r="C20" s="29" t="inlineStr">
-        <is>
-          <t>Desk asked for more metrics based on the research literature; every measure names its source in NB07 and the report references section.</t>
-        </is>
-      </c>
-      <c r="D20" s="29" t="inlineStr">
-        <is>
-          <t>NB07 part A; RESEARCH_REPORT 6.9 + references 8-14</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
mid term presentation v2
</commit_message>
<xml_diff>
--- a/docs/DECISIONS.xlsx
+++ b/docs/DECISIONS.xlsx
@@ -4098,7 +4098,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E64"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="12" min="1" max="1"/>
@@ -5733,7 +5733,34 @@
       </c>
       <c r="E64" s="35" t="inlineStr">
         <is>
-          <t>ADOPTED 2026-07-29; THRESHOLD RE-FIT PENDING - run `python -m analytics.run_analytics --what phases --research`. Offline projection at 54d: threshold ~0.6186, capture 22/98, FA 10 (0.086/inst-yr), AP 0.615 vs 0.608 base, AUROC 0.507, warning 9d. RECORDED COST: the walk-forward loses its 2020 test year, denominator 122 -&gt; 98 - fewer captures REPORTED because it is examined on less, not because it got worse. NOISE: 21 vs 22 of 93 is one episode; 54d sits two steps from the 50d cliff.</t>
+          <t>ADOPTED 2026-07-29; THRESHOLD RE-FIT DONE 2026-07-29: threshold 0.618064, capture 22/98, FA 10 (0.083/inst-yr), AP 0.615 vs 0.608 base, AUROC 0.507, warning 9d - the offline projection was exact. RECORDED COST: the walk-forward loses its 2020 test year, denominator 122 -&gt; 98 - fewer captures REPORTED because it is examined on less, not because it got worse. NOISE: 21 vs 22 of 93 is one episode; 54d sits two steps from the 50d cliff.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="34" t="inlineStr">
+        <is>
+          <t>KNOB AUDIT: every chosen number swept; GET IN brought inside its false-alarm budget; four knobs tested and KEPT</t>
+        </is>
+      </c>
+      <c r="B65" s="35" t="inlineStr">
+        <is>
+          <t>EUPHORIA_ONSET_HYPE_MIN = 1.10 (was a hardcoded 1.0 in desk_candidacy). A1 hype multiple 2.0, A2 attention gate 0.90, GET OUT cooldown 21d and desk trigger smoothing ROLL=7 all swept and left unchanged.</t>
+        </is>
+      </c>
+      <c r="C65" s="35" t="inlineStr">
+        <is>
+          <t>DESK REQUEST 2026-07-29: 'any variables that were arbitrarily defined, we MUST do a frontier on it to determine BEST'. GET IN had breached its own accepted FA budget since it shipped (0.255 vs 0.23), carried as a stated limitation rather than fixed. Floor 1.10 is the max-capture point INSIDE the budget: FA/inst-yr 0.278 -&gt; 0.207, late starts 6 -&gt; 2, precision 0.138 -&gt; 0.173, one capture given up.</t>
+        </is>
+      </c>
+      <c r="D65" s="35" t="inlineStr">
+        <is>
+          <t>Swept on the NB07 A3c frontier: same walk-forward, GROUND TRUTH HELD FIXED (G1/G2/G3, the 120d ground-truth window, the [peak-30d,peak+1d] hit window and the 45d judgeable horizon are all out of scope - tuning them moves the target). KEPT: A1 hype 2.0 IS the capture maximum (22 vs 16-18 either side); A2 att gate 0.90 - monotone trade, nothing inside budget; ROLL 5 weakly dominates 7 by TWO false alarms = noise. COOLDOWN 7d REFUSED despite winning on the stated rule (25 captures vs 22, inside budget) because it fires 78 alerts vs 42 at precision 0.32 - repeat shots at the SAME peak, which the capture count cannot see.</t>
+        </is>
+      </c>
+      <c r="E65" s="35" t="inlineStr">
+        <is>
+          <t>ADOPTED 2026-07-29; RE-FIT PENDING - run `python -m analytics.run_analytics --what phases --research`. COST STATED: 1.0 was a DEFINITION (multiplier one, parameter-free); 1.10 is a fitted number and the register gains an entry it did not have. SCOPE: desk_candidacy only - the crowd-only onset store keeps 1.0 (separate detector, separate record, not swept). OVERFITTING GUARD: six knobs against ~98-125 peaks over a handful of years; nothing adopted on a single-point maximum, only on a stated failure or a broad plateau.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ML Model semi complete - can be tuned more
</commit_message>
<xml_diff>
--- a/docs/DECISIONS.xlsx
+++ b/docs/DECISIONS.xlsx
@@ -23,6 +23,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10. Limitations" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11. Next Steps" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12. References" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13. Aug-2026 Rebuild" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -3215,6 +3216,209 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" style="13" min="1" max="1"/>
+    <col width="70" customWidth="1" style="13" min="2" max="2"/>
+    <col width="60" customWidth="1" style="13" min="3" max="3"/>
+    <col width="10" customWidth="1" style="13" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>13. The August-2026 rebuild - robust shares, swept ground truth, the learned desk model, the presentation pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Evidence / where recorded</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Share-of-chatter estimator rebuilt: trailing-week ratio-of-sums + per-source stratification (90d volume weights) + empirical-Bayes shrinkage (prior strength = MIN_TOTAL). No imputation. Consumed by charts AND signal features.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>analytics/robust_share.py; docs/research/DATA_QUALITY_2026-08.md; notebook 00. Measured: fake zero-days 308-&gt;31 (top-30, May-Aug 2026).</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>SHIPPED</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ground-truth bars lowered: boom 25/50 -&gt; 20/40, bust 15/30 -&gt; 12/25, after a 3-level sweep re-running the full walk-forward per level. 15/30 rejected (episode inflation).</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>PARAMETER_REGISTER Class 14b; docs/research/ml_tournament.json (ground_truth_sweep); notebook 01 SS.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>SHIPPED</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Desk GET IN / GET OUT scored by the tournament winner: logit + monotone-GBM rank ensemble on 9 crowd + 2 price features; candidacy = coverage floor only; operating point = train-year episode F1; 21d cooldown. Pre-stated selection rule: one family both heads, combined test-AP lift.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>analytics/ml_detector.py; notebook 03 SS/SS2; docs/research/ml_tournament.md; euphoria_desk_report.json (carries the full table). GET OUT 42% capture @0.35 FA/iy (rules 12%); GET IN 57% @0.24 (rules 9%).</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SHIPPED</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PM-trust coherence kept under every model: no GET IN on an end-stage day, none within one cooldown after a GET OUT - enforced at the display layer, unit-tested.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>euphoria_phases.rebuild_phase_files; tests TestMLDetector.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>SHIPPED</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>AI Pulse: both score numbers removed (LLM mood gauge X/100 + slider bullishness percentile), including the prompt spec. Tripwire tests added.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>dashboard.py; analytics/ai_pulse.py; tests TestMoodGauge.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>SHIPPED</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Notebook pipeline reshaped to mirror the presentation: 00 data -&gt; 01 ground truth -&gt; 02 features -&gt; 03 tournament -&gt; 04 evaluation -&gt; 05 influence -&gt; 06 worked example (gold) -&gt; 11 presentation pack. Old 00/06/07/08/09/10 retired with frozen JSONs kept live (nb10's AI-sentiment verdict still pending a desk-machine run).</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>notebooks/_retired_2026-08-07_presentation_refactor/README.md; RUNBOOK notebook row.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>SHIPPED</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Crowd-only research detectors unchanged in construction; record re-frozen under the new ground truth (capture 14% of detectable at 0.18 FA/iy) - the 'crowd alone' claim keeps its own honest record beside the desk model.</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>analytics/euphoria.py; euphoria_report.json.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>SHIPPED</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">

</xml_diff>